<commit_message>
Update NPI Dashboard 2026-10-08 13:12
</commit_message>
<xml_diff>
--- a/npi_dashboard.xlsx
+++ b/npi_dashboard.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="NPI Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NPI Dashboard" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'NPI Dashboard'!$A$1:$P$58</definedName>
@@ -3736,7 +3736,7 @@
       </c>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>2027/11/04</t>
+          <t>2026/11/04</t>
         </is>
       </c>
       <c r="J42" s="4" t="inlineStr">
@@ -3769,7 +3769,11 @@
           <t>0A layout中，预计10/26出图</t>
         </is>
       </c>
-      <c r="P42" s="6" t="inlineStr"/>
+      <c r="P42" s="6" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -4082,12 +4086,13 @@
       </c>
       <c r="O46" s="6" t="inlineStr">
         <is>
-          <t>DVT板子測試中, 0N Layout web已開,預計10/14 gerber out.</t>
+          <t>1) DVT板子測試中,SA DP2.1無法測試問題已經跟GRL預約10/7讓SA &amp; EE一起過去GRL debug.
+2) 0N layout進行中,預計10/14 gerber out.</t>
         </is>
       </c>
       <c r="P46" s="6" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>1) 1851 Titan &amp; Raider取消原本 91.8Wh 的規劃，全系列統一採用 99Wh 電池，新開的99Wh電池開模與備料趕不上 1851 EVT，EVT 試產keep採用原本開案規劃的91.8Wh 電池，後續請電池廠商提供手工模樣品for ME RD於 MVT 前進行初步替換驗證.</t>
         </is>
       </c>
     </row>
@@ -4162,12 +4167,13 @@
       </c>
       <c r="O47" s="11" t="inlineStr">
         <is>
-          <t>DVT板子測試中, 0N Layout web已開,預計10/14 gerber out.</t>
+          <t>1) DVT板子測試中,SA DP2.1無法測試問題已經跟GRL預約10/7讓SA &amp; EE一起過去GRL debug.
+2) 0N layout進行中,預計10/14 gerber out.</t>
         </is>
       </c>
       <c r="P47" s="11" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>1) 1851 Titan &amp; Raider取消原本 91.8Wh 的規劃，全系列統一採用 99Wh 電池，新開的99Wh電池開模與備料趕不上 1851 EVT，EVT 試產keep採用原本開案規劃的91.8Wh 電池，後續請電池廠商提供手工模樣品for ME RD於 MVT 前進行初步替換驗證.</t>
         </is>
       </c>
     </row>
@@ -4242,12 +4248,13 @@
       </c>
       <c r="O48" s="11" t="inlineStr">
         <is>
-          <t>DVT板子測試中, 0N Layout web已開,預計10/14 gerber out.</t>
+          <t>1) DVT板子測試中,SA DP2.1無法測試問題已經跟GRL預約10/7讓SA &amp; EE一起過去GRL debug.
+2) 0N layout進行中,預計10/14 gerber out.</t>
         </is>
       </c>
       <c r="P48" s="11" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>1) 1851 Titan &amp; Raider取消原本 91.8Wh 的規劃，全系列統一採用 99Wh 電池，新開的99Wh電池開模與備料趕不上 1851 EVT，EVT 試產keep採用原本開案規劃的91.8Wh 電池，後續請電池廠商提供手工模樣品for ME RD於 MVT 前進行初步替換驗證.</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4279,7 @@
       </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>NVL-HX 65W</t>
+          <t>NVL-HX 55W</t>
         </is>
       </c>
       <c r="F49" s="9" t="inlineStr">
@@ -4322,12 +4329,13 @@
       </c>
       <c r="O49" s="11" t="inlineStr">
         <is>
-          <t>DVT板子測試中, 0N Layout web已開,預計10/14 gerber out.</t>
+          <t>1) DVT板子測試中,SA DP2.1無法測試問題已經跟GRL預約10/7讓SA &amp; EE一起過去GRL debug.
+2) 0N layout進行中,預計10/14 gerber out.</t>
         </is>
       </c>
       <c r="P49" s="11" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>1) 1851 Titan &amp; Raider取消原本 91.8Wh 的規劃，全系列統一採用 99Wh 電池，新開的99Wh電池開模與備料趕不上 1851 EVT，EVT 試產keep採用原本開案規劃的91.8Wh 電池，後續請電池廠商提供手工模樣品for ME RD於 MVT 前進行初步替換驗證.</t>
         </is>
       </c>
     </row>
@@ -4352,7 +4360,7 @@
       </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
-          <t>NVL-HX 65W</t>
+          <t>NVL-HX 55W</t>
         </is>
       </c>
       <c r="F50" s="9" t="inlineStr">
@@ -4402,12 +4410,13 @@
       </c>
       <c r="O50" s="11" t="inlineStr">
         <is>
-          <t>DVT板子測試中, 0N Layout web已開,預計10/14 gerber out.</t>
+          <t>1) DVT板子測試中,SA DP2.1無法測試問題已經跟GRL預約10/7讓SA &amp; EE一起過去GRL debug.
+2) 0N layout進行中,預計10/14 gerber out.</t>
         </is>
       </c>
       <c r="P50" s="11" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>1) 1851 Titan &amp; Raider取消原本 91.8Wh 的規劃，全系列統一採用 99Wh 電池，新開的99Wh電池開模與備料趕不上 1851 EVT，EVT 試產keep採用原本開案規劃的91.8Wh 電池，後續請電池廠商提供手工模樣品for ME RD於 MVT 前進行初步替換驗證.</t>
         </is>
       </c>
     </row>
@@ -4432,7 +4441,7 @@
       </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
-          <t>NVL-HX 65W</t>
+          <t>NVL-HX 55W</t>
         </is>
       </c>
       <c r="F51" s="9" t="inlineStr">
@@ -4482,12 +4491,13 @@
       </c>
       <c r="O51" s="11" t="inlineStr">
         <is>
-          <t>DVT板子測試中, 0N Layout web已開,預計10/14 gerber out.</t>
+          <t>1) DVT板子測試中,SA DP2.1無法測試問題已經跟GRL預約10/7讓SA &amp; EE一起過去GRL debug.
+2) 0N layout進行中,預計10/14 gerber out.</t>
         </is>
       </c>
       <c r="P51" s="11" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>1) 1851 Titan &amp; Raider取消原本 91.8Wh 的規劃，全系列統一採用 99Wh 電池，新開的99Wh電池開模與備料趕不上 1851 EVT，EVT 試產keep採用原本開案規劃的91.8Wh 電池，後續請電池廠商提供手工模樣品for ME RD於 MVT 前進行初步替換驗證.</t>
         </is>
       </c>
     </row>
@@ -4562,7 +4572,7 @@
       </c>
       <c r="O52" s="6" t="inlineStr">
         <is>
-          <t>plan 9/27 EVT SMT，9/28 Pre Assy，10/9 Assy</t>
+          <t>9/27 EVT SMT，9/28 Pre Assy，10/9 Assy</t>
         </is>
       </c>
       <c r="P52" s="6" t="inlineStr">
@@ -4642,7 +4652,7 @@
       </c>
       <c r="O53" s="11" t="inlineStr">
         <is>
-          <t>plan 9/27 EVT SMT，9/28 Pre Assy，10/9 Assy</t>
+          <t>9/27 EVT SMT，9/28 Pre Assy，10/9 Assy</t>
         </is>
       </c>
       <c r="P53" s="11" t="inlineStr">
@@ -4722,7 +4732,7 @@
       </c>
       <c r="O54" s="11" t="inlineStr">
         <is>
-          <t>plan 9/27 EVT SMT，9/28 Pre Assy，10/9 Assy</t>
+          <t>9/27 EVT SMT，9/28 Pre Assy，10/9 Assy</t>
         </is>
       </c>
       <c r="P54" s="11" t="inlineStr">
@@ -4802,7 +4812,7 @@
       </c>
       <c r="O55" s="11" t="inlineStr">
         <is>
-          <t>plan 9/27 EVT SMT，9/28 Pre Assy，10/9 Assy</t>
+          <t>9/27 EVT SMT，9/28 Pre Assy，10/9 Assy</t>
         </is>
       </c>
       <c r="P55" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Update NPI Dashboard 2026-10-13 09:16
</commit_message>
<xml_diff>
--- a/npi_dashboard.xlsx
+++ b/npi_dashboard.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NPI Dashboard" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'NPI Dashboard'!$A$1:$P$58</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'NPI Dashboard'!$A$1:$P$59</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -511,7 +511,7 @@
     <outlinePr summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P58"/>
+  <dimension ref="A1:P59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -677,9 +677,8 @@
       </c>
       <c r="O2" s="6" t="inlineStr">
         <is>
-          <t>(
-1).8/19 Resume並新增new CPU R7 9800HX3D. (
-2). CPU缺料,9/15-16 MVT齊料.</t>
+          <t>1).8/19 Resume並新增new CPU R7 9800HX3D
+2).MVT測試中</t>
         </is>
       </c>
       <c r="P2" s="6" t="inlineStr">
@@ -751,9 +750,8 @@
       </c>
       <c r="O3" s="11" t="inlineStr">
         <is>
-          <t>(
-1).8/19 Resume並新增new CPU R7 9800HX3D. (
-2). CPU缺料,9/15-16 MVT齊料.</t>
+          <t>1).8/19 Resume並新增new CPU R7 9800HX3D
+2).MVT測試中</t>
         </is>
       </c>
       <c r="P3" s="11" t="inlineStr">
@@ -825,9 +823,8 @@
       </c>
       <c r="O4" s="11" t="inlineStr">
         <is>
-          <t>(
-1).8/19 Resume並新增new CPU R7 9800HX3D. (
-2). CPU缺料,9/15-16 MVT齊料.</t>
+          <t>1).8/19 Resume並新增new CPU R7 9800HX3D
+2).MVT測試中</t>
         </is>
       </c>
       <c r="P4" s="11" t="inlineStr">
@@ -912,8 +909,8 @@
       </c>
       <c r="P5" s="6" t="inlineStr">
         <is>
-          <t>1)備料：a. 2.8K panel: MP*1K交期, 9/23 SDC update因PCB物料短缺, 會delay至11/M ETD,仍在請廠商pull in中  b. PCB: 9/23 1.0出圖, 只先備料300 pcs for ATS use.
-2）Issue: N1 performance limit around 40W, 影響PCB risk buy, target 2 weeks 10/9之前釐清問題</t>
+          <t>1)備料：a. 2.8K panel: SDC update因PCB物料短缺會delay至11/M ETD, 影響2nd MP時間約1 week , 仍在請廠商pull in中  b. PCB: 1.0 Gerber out@9/23, 9/23備料600 pcs, 10/6確定可備料2.4k for 2nd MP.
+2）Issue: 10/12-10/16 PM&amp;RD至NV on-site debug</t>
         </is>
       </c>
     </row>
@@ -1068,7 +1065,7 @@
       </c>
       <c r="O7" s="6" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR5: MVT SMT @ 10/12, Pre-assy @ 10/14, Assy @ 10/16</t>
+          <t>RPL-HX R + DDR5: MVT SMT @ 10/13, Pre-assy @ 10/14, Assy @ 10/16</t>
         </is>
       </c>
       <c r="P7" s="6" t="inlineStr">
@@ -1148,7 +1145,7 @@
       </c>
       <c r="O8" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR5: MVT SMT @ 10/12, Pre-assy @ 10/14, Assy @ 10/16</t>
+          <t>RPL-HX R + DDR5: MVT SMT @ 10/13, Pre-assy @ 10/14, Assy @ 10/16</t>
         </is>
       </c>
       <c r="P8" s="11" t="inlineStr">
@@ -1228,7 +1225,7 @@
       </c>
       <c r="O9" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR5: MVT SMT @ 10/12, Pre-assy @ 10/14, Assy @ 10/16</t>
+          <t>RPL-HX R + DDR5: MVT SMT @ 10/13, Pre-assy @ 10/14, Assy @ 10/16</t>
         </is>
       </c>
       <c r="P9" s="11" t="inlineStr">
@@ -1308,7 +1305,7 @@
       </c>
       <c r="O10" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR5: MVT SMT @ 10/12, Pre-assy @ 10/14, Assy @ 10/16</t>
+          <t>RPL-HX R + DDR5: MVT SMT @ 10/13, Pre-assy @ 10/14, Assy @ 10/16</t>
         </is>
       </c>
       <c r="P10" s="11" t="inlineStr">
@@ -2572,12 +2569,13 @@
       </c>
       <c r="O27" s="6" t="inlineStr">
         <is>
-          <t>EVT SMT@9/16</t>
+          <t>DQA 測試中</t>
         </is>
       </c>
       <c r="P27" s="6" t="inlineStr">
         <is>
-          <t>1) Schedule:NV VBIOS @1/6, gating 8天,預計12/E 拿到WHQL，可能影響到最終TTM 時間</t>
+          <t>1)S1J-AE6C002-TH1 Panel 在 NVL-H平台 無法調亮度,已經請Intel 協助;
+2) Schedule:NV VBIOS @1/6, gating 8天,預計12/E 拿到WHQL，可能影響到最終TTM 時間</t>
         </is>
       </c>
     </row>
@@ -2652,7 +2650,7 @@
       </c>
       <c r="O28" s="11" t="inlineStr">
         <is>
-          <t>EVT SMT@9/16</t>
+          <t>DQA 測試中</t>
         </is>
       </c>
       <c r="P28" s="11" t="inlineStr">
@@ -2732,7 +2730,7 @@
       </c>
       <c r="O29" s="11" t="inlineStr">
         <is>
-          <t>EVT SMT@9/16</t>
+          <t>DQA 測試中</t>
         </is>
       </c>
       <c r="P29" s="11" t="inlineStr">
@@ -2818,7 +2816,8 @@
       <c r="P30" s="6" t="inlineStr">
         <is>
           <t>1)NV VBIOS 驗證時間6周
-2)Intel WHQL :12/E 拿到 可能影響到最終TTM 時間</t>
+2)Intel WHQL :12/E 拿到 可能影響到最終TTM 時間
+3)備料: OLED panel 因無法調亮度問題目前還在找對策,可能影響出貨</t>
         </is>
       </c>
     </row>
@@ -2899,7 +2898,8 @@
       <c r="P31" s="11" t="inlineStr">
         <is>
           <t>1)NV VBIOS 驗證時間6周
-2)Intel WHQL :12/E 拿到 可能影響到最終TTM 時間</t>
+2)Intel WHQL :12/E 拿到 可能影響到最終TTM 時間
+3)備料: OLED panel 因無法調亮度問題目前還在找對策,可能影響出貨</t>
         </is>
       </c>
     </row>
@@ -2980,7 +2980,8 @@
       <c r="P32" s="11" t="inlineStr">
         <is>
           <t>1)NV VBIOS 驗證時間6周
-2)Intel WHQL :12/E 拿到 可能影響到最終TTM 時間</t>
+2)Intel WHQL :12/E 拿到 可能影響到最終TTM 時間
+3)備料: OLED panel 因無法調亮度問題目前還在找對策,可能影響出貨</t>
         </is>
       </c>
     </row>
@@ -3061,7 +3062,8 @@
       <c r="P33" s="11" t="inlineStr">
         <is>
           <t>1)NV VBIOS 驗證時間6周
-2)Intel WHQL :12/E 拿到 可能影響到最終TTM 時間</t>
+2)Intel WHQL :12/E 拿到 可能影響到最終TTM 時間
+3)備料: OLED panel 因無法調亮度問題目前還在找對策,可能影響出貨</t>
         </is>
       </c>
     </row>
@@ -5061,8 +5063,80 @@
         </is>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>2665</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>Cyborg N16 C1M</t>
+        </is>
+      </c>
+      <c r="D59" s="16" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="inlineStr">
+        <is>
+          <t>N1 45W</t>
+        </is>
+      </c>
+      <c r="F59" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G59" s="4" t="inlineStr">
+        <is>
+          <t>梅燕</t>
+        </is>
+      </c>
+      <c r="H59" s="4" t="inlineStr">
+        <is>
+          <t>2026/09/30</t>
+        </is>
+      </c>
+      <c r="I59" s="4" t="inlineStr">
+        <is>
+          <t>2026/11/25</t>
+        </is>
+      </c>
+      <c r="J59" s="4" t="inlineStr">
+        <is>
+          <t>2026/12/16</t>
+        </is>
+      </c>
+      <c r="K59" s="4" t="inlineStr">
+        <is>
+          <t>2027/02/24</t>
+        </is>
+      </c>
+      <c r="L59" s="4" t="inlineStr">
+        <is>
+          <t>2027/03/01</t>
+        </is>
+      </c>
+      <c r="M59" s="4" t="inlineStr">
+        <is>
+          <t>2027/03/27</t>
+        </is>
+      </c>
+      <c r="N59" s="4" t="inlineStr">
+        <is>
+          <t>2027/04/09</t>
+        </is>
+      </c>
+      <c r="O59" s="6" t="inlineStr"/>
+      <c r="P59" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P58"/>
+  <autoFilter ref="A1:P59"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update NPI Dashboard 2026-10-15 13:14
</commit_message>
<xml_diff>
--- a/npi_dashboard.xlsx
+++ b/npi_dashboard.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NPI Dashboard" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'NPI Dashboard'!$A$1:$P$59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'NPI Dashboard'!$A$1:$P$62</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -511,7 +511,7 @@
     <outlinePr summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P59"/>
+  <dimension ref="A1:P62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -620,12 +620,12 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>265K</t>
+          <t>15T2</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Raider A16 HX B9WI</t>
+          <t>Cyborg 15 C3M</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
@@ -635,126 +635,121 @@
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>FRG-HX3D 55W</t>
+          <t>PTL-H 80W</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>RTX 5080</t>
+          <t>Intel® Arc™ Graphics</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>梅燕</t>
+          <t>李文欽</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>2025/10/15</t>
+          <t>2026/10/13</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr"/>
       <c r="J2" s="4" t="inlineStr"/>
-      <c r="K2" s="4" t="inlineStr">
+      <c r="K2" s="4" t="inlineStr"/>
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t>2026/10/20</t>
+        </is>
+      </c>
+      <c r="M2" s="4" t="inlineStr">
+        <is>
+          <t>2026/11/02</t>
+        </is>
+      </c>
+      <c r="N2" s="4" t="inlineStr">
+        <is>
+          <t>2026/11/15</t>
+        </is>
+      </c>
+      <c r="O2" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P2" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>265K</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Raider A16 HX B9WI</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>MVT</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>FRG-HX3D 55W</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>RTX 5080</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>梅燕</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>2025/10/15</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr"/>
+      <c r="J3" s="4" t="inlineStr"/>
+      <c r="K3" s="4" t="inlineStr">
         <is>
           <t>2026/09/18</t>
         </is>
       </c>
-      <c r="L2" s="4" t="inlineStr">
+      <c r="L3" s="4" t="inlineStr">
         <is>
           <t>2026/10/12</t>
         </is>
       </c>
-      <c r="M2" s="4" t="inlineStr">
+      <c r="M3" s="4" t="inlineStr">
         <is>
           <t>2026/11/06</t>
         </is>
       </c>
-      <c r="N2" s="4" t="inlineStr">
+      <c r="N3" s="4" t="inlineStr">
         <is>
           <t>2026/11/16</t>
         </is>
       </c>
-      <c r="O2" s="6" t="inlineStr">
+      <c r="O3" s="6" t="inlineStr">
         <is>
           <t>1).8/19 Resume並新增new CPU R7 9800HX3D
 2).MVT測試中</t>
         </is>
       </c>
-      <c r="P2" s="6" t="inlineStr">
-        <is>
-          <t>無.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" hidden="1" outlineLevel="1">
-      <c r="A3" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>265K</t>
-        </is>
-      </c>
-      <c r="C3" s="9" t="inlineStr">
-        <is>
-          <t>Raider A16 HX B9WJ</t>
-        </is>
-      </c>
-      <c r="D3" s="10" t="inlineStr">
-        <is>
-          <t>MVT</t>
-        </is>
-      </c>
-      <c r="E3" s="9" t="inlineStr">
-        <is>
-          <t>FRG-HX3D 55W</t>
-        </is>
-      </c>
-      <c r="F3" s="9" t="inlineStr">
-        <is>
-          <t>RTX 5090</t>
-        </is>
-      </c>
-      <c r="G3" s="9" t="inlineStr">
-        <is>
-          <t>梅燕</t>
-        </is>
-      </c>
-      <c r="H3" s="9" t="inlineStr">
-        <is>
-          <t>2025/10/15</t>
-        </is>
-      </c>
-      <c r="I3" s="9" t="inlineStr"/>
-      <c r="J3" s="9" t="inlineStr"/>
-      <c r="K3" s="9" t="inlineStr">
-        <is>
-          <t>2026/09/18</t>
-        </is>
-      </c>
-      <c r="L3" s="9" t="inlineStr">
-        <is>
-          <t>2026/10/12</t>
-        </is>
-      </c>
-      <c r="M3" s="9" t="inlineStr">
-        <is>
-          <t>2026/11/06</t>
-        </is>
-      </c>
-      <c r="N3" s="9" t="inlineStr">
-        <is>
-          <t>2026/11/16</t>
-        </is>
-      </c>
-      <c r="O3" s="11" t="inlineStr">
-        <is>
-          <t>1).8/19 Resume並新增new CPU R7 9800HX3D
-2).MVT測試中</t>
-        </is>
-      </c>
-      <c r="P3" s="11" t="inlineStr">
+      <c r="P3" s="6" t="inlineStr">
         <is>
           <t>無.</t>
         </is>
@@ -771,7 +766,7 @@
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>Raider A16 HX B9WH</t>
+          <t>Raider A16 HX B9WJ</t>
         </is>
       </c>
       <c r="D4" s="10" t="inlineStr">
@@ -786,7 +781,7 @@
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>RTX 5070Ti</t>
+          <t>RTX 5090</t>
         </is>
       </c>
       <c r="G4" s="9" t="inlineStr">
@@ -829,88 +824,80 @@
       </c>
       <c r="P4" s="11" t="inlineStr">
         <is>
+          <t>無.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" hidden="1" outlineLevel="1">
+      <c r="A5" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>265K</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>Raider A16 HX B9WH</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>MVT</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>FRG-HX3D 55W</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>RTX 5070Ti</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>梅燕</t>
+        </is>
+      </c>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>2025/10/15</t>
+        </is>
+      </c>
+      <c r="I5" s="9" t="inlineStr"/>
+      <c r="J5" s="9" t="inlineStr"/>
+      <c r="K5" s="9" t="inlineStr">
+        <is>
+          <t>2026/09/18</t>
+        </is>
+      </c>
+      <c r="L5" s="9" t="inlineStr">
+        <is>
+          <t>2026/10/12</t>
+        </is>
+      </c>
+      <c r="M5" s="9" t="inlineStr">
+        <is>
+          <t>2026/11/06</t>
+        </is>
+      </c>
+      <c r="N5" s="9" t="inlineStr">
+        <is>
+          <t>2026/11/16</t>
+        </is>
+      </c>
+      <c r="O5" s="11" t="inlineStr">
+        <is>
+          <t>1).8/19 Resume並新增new CPU R7 9800HX3D
+2).MVT測試中</t>
+        </is>
+      </c>
+      <c r="P5" s="11" t="inlineStr">
+        <is>
           <t>無</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>14T3</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>Prestige N14 AI+ D1M</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>MVT</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>N1 35W</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>倪嬌嬌</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>2025/04/30</t>
-        </is>
-      </c>
-      <c r="I5" s="4" t="inlineStr">
-        <is>
-          <t>2025/09/01</t>
-        </is>
-      </c>
-      <c r="J5" s="4" t="inlineStr">
-        <is>
-          <t>2026/04/15</t>
-        </is>
-      </c>
-      <c r="K5" s="4" t="inlineStr">
-        <is>
-          <t>2026/08/13</t>
-        </is>
-      </c>
-      <c r="L5" s="4" t="inlineStr">
-        <is>
-          <t>2026/09/16</t>
-        </is>
-      </c>
-      <c r="M5" s="4" t="inlineStr">
-        <is>
-          <t>2026/11/09</t>
-        </is>
-      </c>
-      <c r="N5" s="4" t="inlineStr">
-        <is>
-          <t>2026/11/23</t>
-        </is>
-      </c>
-      <c r="O5" s="6" t="inlineStr">
-        <is>
-          <t>MVT DQA test中, 1.0 Gerber out@9/23--先備料300 pcs for ATS use</t>
-        </is>
-      </c>
-      <c r="P5" s="6" t="inlineStr">
-        <is>
-          <t>1)備料：a. 2.8K panel: SDC update因PCB物料短缺會delay至11/M ETD, 影響2nd MP時間約1 week , 仍在請廠商pull in中  b. PCB: 1.0 Gerber out@9/23, 9/23備料600 pcs, 10/6確定可備料2.4k for 2nd MP.
-2）Issue: 10/12-10/16 PM&amp;RD至NV on-site debug</t>
         </is>
       </c>
     </row>
@@ -920,12 +907,12 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>2623</t>
+          <t>14T3</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Prestige N16 AI+ C1M</t>
+          <t>Prestige N14 AI+ D1M</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -935,7 +922,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>N1 45W</t>
+          <t>N1 35W</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -945,7 +932,7 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>賴雪鳳</t>
+          <t>倪嬌嬌</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
@@ -970,7 +957,7 @@
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>2026/09/14</t>
+          <t>2026/09/16</t>
         </is>
       </c>
       <c r="M6" s="4" t="inlineStr">
@@ -985,12 +972,13 @@
       </c>
       <c r="O6" s="6" t="inlineStr">
         <is>
-          <t>機台已經全數回台,並分寄給NV  MVT驗證中</t>
+          <t>MVT DQA test中, 1.0 Gerber out@9/23--先備料300 pcs for ATS use</t>
         </is>
       </c>
       <c r="P6" s="6" t="inlineStr">
         <is>
-          <t>備料: Samsung 2.8K panel 採購備料HR14*2K for N1 ATS 用, 另外要再驗證HR16 for後續出貨需求</t>
+          <t>1)備料：a. 2.8K panel: SDC update因PCB物料短缺會delay至11/M ETD, 影響2nd MP時間約1 week , 仍在請廠商pull in中  b. PCB: 1.0 Gerber out@9/23, 9/23備料600 pcs, 10/6確定可備料2.4k for 2nd MP.
+2）Issue: 10/12-10/16 PM&amp;RD至NV on-site debug</t>
         </is>
       </c>
     </row>
@@ -1000,155 +988,155 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
+          <t>2623</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Prestige N16 AI+ C1M</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>MVT</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>N1 45W</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>賴雪鳳</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>2025/04/30</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>2025/09/01</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>2026/04/15</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>2026/08/13</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>2026/09/14</t>
+        </is>
+      </c>
+      <c r="M7" s="4" t="inlineStr">
+        <is>
+          <t>2026/11/09</t>
+        </is>
+      </c>
+      <c r="N7" s="4" t="inlineStr">
+        <is>
+          <t>2026/11/23</t>
+        </is>
+      </c>
+      <c r="O7" s="6" t="inlineStr">
+        <is>
+          <t>機台已經全數回台,並分寄給NV  MVT驗證中</t>
+        </is>
+      </c>
+      <c r="P7" s="6" t="inlineStr">
+        <is>
+          <t>備料: Samsung 2.8K panel 採購備料HR14*2K for N1 ATS 用, 另外要再驗證HR16 for後續出貨需求</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
           <t>1861</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>Katana 18 HX A14WEK</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>MVT</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>RPL-HX refresh 55W</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>RTX 5050</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>顧曉琴</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="H8" s="4" t="inlineStr">
         <is>
           <t>2026/05/08</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="I8" s="4" t="inlineStr">
         <is>
           <t>2026/06/15</t>
         </is>
       </c>
-      <c r="J7" s="4" t="inlineStr">
+      <c r="J8" s="4" t="inlineStr">
         <is>
           <t>2026/08/13</t>
         </is>
       </c>
-      <c r="K7" s="4" t="inlineStr">
+      <c r="K8" s="4" t="inlineStr">
         <is>
           <t>2026/10/12</t>
         </is>
       </c>
-      <c r="L7" s="4" t="inlineStr">
+      <c r="L8" s="4" t="inlineStr">
         <is>
           <t>2026/11/02</t>
         </is>
       </c>
-      <c r="M7" s="4" t="inlineStr">
+      <c r="M8" s="4" t="inlineStr">
         <is>
           <t>2026/11/21</t>
         </is>
       </c>
-      <c r="N7" s="4" t="inlineStr">
+      <c r="N8" s="4" t="inlineStr">
         <is>
           <t>2026/11/30</t>
         </is>
       </c>
-      <c r="O7" s="6" t="inlineStr">
-        <is>
-          <t>RPL-HX R + DDR5: MVT SMT @ 10/13, Pre-assy @ 10/14, Assy @ 10/16</t>
-        </is>
-      </c>
-      <c r="P7" s="6" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" hidden="1" outlineLevel="1">
-      <c r="A8" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>1861</t>
-        </is>
-      </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>Katana 18 HX A14WFK</t>
-        </is>
-      </c>
-      <c r="D8" s="10" t="inlineStr">
-        <is>
-          <t>MVT</t>
-        </is>
-      </c>
-      <c r="E8" s="9" t="inlineStr">
-        <is>
-          <t>RPL-HX refresh 55W</t>
-        </is>
-      </c>
-      <c r="F8" s="9" t="inlineStr">
-        <is>
-          <t>RTX 5060</t>
-        </is>
-      </c>
-      <c r="G8" s="9" t="inlineStr">
-        <is>
-          <t>顧曉琴</t>
-        </is>
-      </c>
-      <c r="H8" s="9" t="inlineStr">
-        <is>
-          <t>2026/05/08</t>
-        </is>
-      </c>
-      <c r="I8" s="9" t="inlineStr">
-        <is>
-          <t>2026/06/15</t>
-        </is>
-      </c>
-      <c r="J8" s="9" t="inlineStr">
-        <is>
-          <t>2026/08/13</t>
-        </is>
-      </c>
-      <c r="K8" s="9" t="inlineStr">
-        <is>
-          <t>2026/10/12</t>
-        </is>
-      </c>
-      <c r="L8" s="9" t="inlineStr">
-        <is>
-          <t>2026/11/02</t>
-        </is>
-      </c>
-      <c r="M8" s="9" t="inlineStr">
-        <is>
-          <t>2026/11/21</t>
-        </is>
-      </c>
-      <c r="N8" s="9" t="inlineStr">
-        <is>
-          <t>2026/11/30</t>
-        </is>
-      </c>
-      <c r="O8" s="11" t="inlineStr">
-        <is>
-          <t>RPL-HX R + DDR5: MVT SMT @ 10/13, Pre-assy @ 10/14, Assy @ 10/16</t>
-        </is>
-      </c>
-      <c r="P8" s="11" t="inlineStr">
+      <c r="O8" s="6" t="inlineStr">
+        <is>
+          <t>RPL-HX R + DDR5: MVT Assy @ 10/16, 預計10/21領取給DQA測試</t>
+        </is>
+      </c>
+      <c r="P8" s="6" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1165,7 +1153,7 @@
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>Katana 18 HX A14WGK</t>
+          <t>Katana 18 HX A14WFK</t>
         </is>
       </c>
       <c r="D9" s="10" t="inlineStr">
@@ -1180,7 +1168,7 @@
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>RTX 5070</t>
+          <t>RTX 5060</t>
         </is>
       </c>
       <c r="G9" s="9" t="inlineStr">
@@ -1225,7 +1213,7 @@
       </c>
       <c r="O9" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR5: MVT SMT @ 10/13, Pre-assy @ 10/14, Assy @ 10/16</t>
+          <t>RPL-HX R + DDR5: MVT Assy @ 10/16, 預計10/21領取給DQA測試</t>
         </is>
       </c>
       <c r="P9" s="11" t="inlineStr">
@@ -1245,7 +1233,7 @@
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Katana 18 HX A14WGXK</t>
+          <t>Katana 18 HX A14WGK</t>
         </is>
       </c>
       <c r="D10" s="10" t="inlineStr">
@@ -1305,7 +1293,7 @@
       </c>
       <c r="O10" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR5: MVT SMT @ 10/13, Pre-assy @ 10/14, Assy @ 10/16</t>
+          <t>RPL-HX R + DDR5: MVT Assy @ 10/16, 預計10/21領取給DQA測試</t>
         </is>
       </c>
       <c r="P10" s="11" t="inlineStr">
@@ -1325,7 +1313,7 @@
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>Katana 18 HX A14WEOK</t>
+          <t>Katana 18 HX A14WGXK</t>
         </is>
       </c>
       <c r="D11" s="10" t="inlineStr">
@@ -1340,7 +1328,7 @@
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>RTX 5050</t>
+          <t>RTX 5070</t>
         </is>
       </c>
       <c r="G11" s="9" t="inlineStr">
@@ -1350,18 +1338,22 @@
       </c>
       <c r="H11" s="9" t="inlineStr">
         <is>
-          <t>2026/05/20</t>
+          <t>2026/05/08</t>
         </is>
       </c>
       <c r="I11" s="9" t="inlineStr">
         <is>
-          <t>2026/06/27</t>
-        </is>
-      </c>
-      <c r="J11" s="9" t="inlineStr"/>
+          <t>2026/06/15</t>
+        </is>
+      </c>
+      <c r="J11" s="9" t="inlineStr">
+        <is>
+          <t>2026/08/13</t>
+        </is>
+      </c>
       <c r="K11" s="9" t="inlineStr">
         <is>
-          <t>2026/10/19</t>
+          <t>2026/10/12</t>
         </is>
       </c>
       <c r="L11" s="9" t="inlineStr">
@@ -1371,22 +1363,22 @@
       </c>
       <c r="M11" s="9" t="inlineStr">
         <is>
-          <t>2026/11/23</t>
+          <t>2026/11/21</t>
         </is>
       </c>
       <c r="N11" s="9" t="inlineStr">
         <is>
-          <t>2026/12/02</t>
+          <t>2026/11/30</t>
         </is>
       </c>
       <c r="O11" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR4: 3.1 G/O @ 9/24, MVT SMT @ 10/19, Pre-assy @ 10/20, Assy @ 10/22</t>
+          <t>RPL-HX R + DDR5: MVT Assy @ 10/16, 預計10/21領取給DQA測試</t>
         </is>
       </c>
       <c r="P11" s="11" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -1401,7 +1393,7 @@
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>Katana 18 HX A14WFOK</t>
+          <t>Katana 18 HX A14WEOK</t>
         </is>
       </c>
       <c r="D12" s="10" t="inlineStr">
@@ -1416,7 +1408,7 @@
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>RTX 5060</t>
+          <t>RTX 5050</t>
         </is>
       </c>
       <c r="G12" s="9" t="inlineStr">
@@ -1457,7 +1449,7 @@
       </c>
       <c r="O12" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR4: 3.1 G/O @ 9/24, MVT SMT @ 10/19, Pre-assy @ 10/20, Assy @ 10/22</t>
+          <t>RPL-HX R + DDR4: MVT SMT @ 10/19, Pre-assy @ 10/20, Assy @ 10/22</t>
         </is>
       </c>
       <c r="P12" s="11" t="inlineStr">
@@ -1477,7 +1469,7 @@
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>Katana 18 HX A14WGOK</t>
+          <t>Katana 18 HX A14WFOK</t>
         </is>
       </c>
       <c r="D13" s="10" t="inlineStr">
@@ -1492,7 +1484,7 @@
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t>RTX 5070</t>
+          <t>RTX 5060</t>
         </is>
       </c>
       <c r="G13" s="9" t="inlineStr">
@@ -1533,7 +1525,7 @@
       </c>
       <c r="O13" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR4:3.1 G/O @ 9/24, MVT SMT @ 10/19, Pre-assy @ 10/20, Assy @ 10/22</t>
+          <t>RPL-HX R + DDR4: MVT SMT @ 10/19, Pre-assy @ 10/20, Assy @ 10/22</t>
         </is>
       </c>
       <c r="P13" s="11" t="inlineStr">
@@ -1553,7 +1545,7 @@
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>Katana 18 HX A14WGXOK</t>
+          <t>Katana 18 HX A14WGOK</t>
         </is>
       </c>
       <c r="D14" s="10" t="inlineStr">
@@ -1609,7 +1601,7 @@
       </c>
       <c r="O14" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR4: 3.1 G/O @ 9/24, MVT SMT @ 10/19, Pre-assy @ 10/20, Assy @ 10/22</t>
+          <t>RPL-HX R + DDR4: MVT SMT @ 10/19, Pre-assy @ 10/20, Assy @ 10/22</t>
         </is>
       </c>
       <c r="P14" s="11" t="inlineStr">
@@ -1629,22 +1621,22 @@
       </c>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t>Katana 18 HX A2WEK</t>
-        </is>
-      </c>
-      <c r="D15" s="12" t="inlineStr">
-        <is>
-          <t>Design</t>
+          <t>Katana 18 HX A14WGXOK</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>MVT</t>
         </is>
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>RPL-HX Next 55W</t>
+          <t>RPL-HX refresh 55W</t>
         </is>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>RTX 5050</t>
+          <t>RTX 5070</t>
         </is>
       </c>
       <c r="G15" s="9" t="inlineStr">
@@ -1654,34 +1646,38 @@
       </c>
       <c r="H15" s="9" t="inlineStr">
         <is>
-          <t>2026/05/08</t>
-        </is>
-      </c>
-      <c r="I15" s="9" t="inlineStr"/>
+          <t>2026/05/20</t>
+        </is>
+      </c>
+      <c r="I15" s="9" t="inlineStr">
+        <is>
+          <t>2026/06/27</t>
+        </is>
+      </c>
       <c r="J15" s="9" t="inlineStr"/>
       <c r="K15" s="9" t="inlineStr">
         <is>
-          <t>2026/12/08</t>
+          <t>2026/10/19</t>
         </is>
       </c>
       <c r="L15" s="9" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/11/02</t>
         </is>
       </c>
       <c r="M15" s="9" t="inlineStr">
         <is>
-          <t>2027/01/19</t>
+          <t>2026/11/23</t>
         </is>
       </c>
       <c r="N15" s="9" t="inlineStr">
         <is>
-          <t>2027/01/30</t>
+          <t>2026/12/02</t>
         </is>
       </c>
       <c r="O15" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX Next + DDR5: follow RPL HX Refresh, 待RPL HX Next QS sample WW49到料後安排MVT</t>
+          <t>RPL-HX R + DDR4: MVT SMT @ 10/19, Pre-assy @ 10/20, Assy @ 10/22</t>
         </is>
       </c>
       <c r="P15" s="11" t="inlineStr">
@@ -1701,7 +1697,7 @@
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>Katana 18 HX A2WEOK</t>
+          <t>Katana 18 HX A2WEK</t>
         </is>
       </c>
       <c r="D16" s="12" t="inlineStr">
@@ -1726,14 +1722,10 @@
       </c>
       <c r="H16" s="9" t="inlineStr">
         <is>
-          <t>2026/05/20</t>
-        </is>
-      </c>
-      <c r="I16" s="9" t="inlineStr">
-        <is>
-          <t>2026/06/27</t>
-        </is>
-      </c>
+          <t>2026/05/08</t>
+        </is>
+      </c>
+      <c r="I16" s="9" t="inlineStr"/>
       <c r="J16" s="9" t="inlineStr"/>
       <c r="K16" s="9" t="inlineStr">
         <is>
@@ -1757,7 +1749,7 @@
       </c>
       <c r="O16" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX Next+ DDR4: follow RPL HX Refresh, 待RPL HX Next QS sample WW49到料後安排MVT</t>
+          <t>RPL-HX Next + DDR5: follow RPL HX Refresh, 待RPL HX Next QS sample WW49到料後安排MVT</t>
         </is>
       </c>
       <c r="P16" s="11" t="inlineStr">
@@ -1777,7 +1769,7 @@
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>Katana 18 HX A2WFK</t>
+          <t>Katana 18 HX A2WEOK</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
@@ -1792,7 +1784,7 @@
       </c>
       <c r="F17" s="9" t="inlineStr">
         <is>
-          <t>RTX 5060</t>
+          <t>RTX 5050</t>
         </is>
       </c>
       <c r="G17" s="9" t="inlineStr">
@@ -1802,10 +1794,14 @@
       </c>
       <c r="H17" s="9" t="inlineStr">
         <is>
-          <t>2026/05/08</t>
-        </is>
-      </c>
-      <c r="I17" s="9" t="inlineStr"/>
+          <t>2026/05/20</t>
+        </is>
+      </c>
+      <c r="I17" s="9" t="inlineStr">
+        <is>
+          <t>2026/06/27</t>
+        </is>
+      </c>
       <c r="J17" s="9" t="inlineStr"/>
       <c r="K17" s="9" t="inlineStr">
         <is>
@@ -1829,7 +1825,7 @@
       </c>
       <c r="O17" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX Next + DDR5: follow RPL HX Refresh, 待RPL HX Next QS sample WW49到料後安排MVT</t>
+          <t>RPL-HX Next+ DDR4: follow RPL HX Refresh, 待RPL HX Next QS sample WW49到料後安排MVT</t>
         </is>
       </c>
       <c r="P17" s="11" t="inlineStr">
@@ -1849,7 +1845,7 @@
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>Katana 18 HX A2WFOK</t>
+          <t>Katana 18 HX A2WFK</t>
         </is>
       </c>
       <c r="D18" s="12" t="inlineStr">
@@ -1874,14 +1870,10 @@
       </c>
       <c r="H18" s="9" t="inlineStr">
         <is>
-          <t>2026/05/20</t>
-        </is>
-      </c>
-      <c r="I18" s="9" t="inlineStr">
-        <is>
-          <t>2026/06/27</t>
-        </is>
-      </c>
+          <t>2026/05/08</t>
+        </is>
+      </c>
+      <c r="I18" s="9" t="inlineStr"/>
       <c r="J18" s="9" t="inlineStr"/>
       <c r="K18" s="9" t="inlineStr">
         <is>
@@ -1905,7 +1897,7 @@
       </c>
       <c r="O18" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX Next+ DDR4: follow RPL HX Refresh, 待RPL HX Next QS sample WW49到料後安排MVT</t>
+          <t>RPL-HX Next + DDR5: follow RPL HX Refresh, 待RPL HX Next QS sample WW49到料後安排MVT</t>
         </is>
       </c>
       <c r="P18" s="11" t="inlineStr">
@@ -1925,7 +1917,7 @@
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>Katana 18 HX A2WGK</t>
+          <t>Katana 18 HX A2WFOK</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
@@ -1940,7 +1932,7 @@
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
-          <t>RTX 5070</t>
+          <t>RTX 5060</t>
         </is>
       </c>
       <c r="G19" s="9" t="inlineStr">
@@ -1950,10 +1942,14 @@
       </c>
       <c r="H19" s="9" t="inlineStr">
         <is>
-          <t>2026/05/08</t>
-        </is>
-      </c>
-      <c r="I19" s="9" t="inlineStr"/>
+          <t>2026/05/20</t>
+        </is>
+      </c>
+      <c r="I19" s="9" t="inlineStr">
+        <is>
+          <t>2026/06/27</t>
+        </is>
+      </c>
       <c r="J19" s="9" t="inlineStr"/>
       <c r="K19" s="9" t="inlineStr">
         <is>
@@ -1977,7 +1973,7 @@
       </c>
       <c r="O19" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX Next + DDR5: follow RPL HX Refresh, 待RPL HX Next QS sample WW49到料後安排MVT</t>
+          <t>RPL-HX Next+ DDR4: follow RPL HX Refresh, 待RPL HX Next QS sample WW49到料後安排MVT</t>
         </is>
       </c>
       <c r="P19" s="11" t="inlineStr">
@@ -1997,7 +1993,7 @@
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>Katana 18 HX A2WGOK</t>
+          <t>Katana 18 HX A2WGK</t>
         </is>
       </c>
       <c r="D20" s="12" t="inlineStr">
@@ -2022,14 +2018,10 @@
       </c>
       <c r="H20" s="9" t="inlineStr">
         <is>
-          <t>2026/05/20</t>
-        </is>
-      </c>
-      <c r="I20" s="9" t="inlineStr">
-        <is>
-          <t>2026/06/27</t>
-        </is>
-      </c>
+          <t>2026/05/08</t>
+        </is>
+      </c>
+      <c r="I20" s="9" t="inlineStr"/>
       <c r="J20" s="9" t="inlineStr"/>
       <c r="K20" s="9" t="inlineStr">
         <is>
@@ -2053,7 +2045,7 @@
       </c>
       <c r="O20" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX Next+ DDR4: follow RPL HX Refresh, 待RPL HX Next QS sample WW49到料後安排MVT</t>
+          <t>RPL-HX Next + DDR5: follow RPL HX Refresh, 待RPL HX Next QS sample WW49到料後安排MVT</t>
         </is>
       </c>
       <c r="P20" s="11" t="inlineStr">
@@ -2073,7 +2065,7 @@
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>Katana 18 HX A2WGXK</t>
+          <t>Katana 18 HX A2WGOK</t>
         </is>
       </c>
       <c r="D21" s="12" t="inlineStr">
@@ -2098,10 +2090,14 @@
       </c>
       <c r="H21" s="9" t="inlineStr">
         <is>
-          <t>2026/05/08</t>
-        </is>
-      </c>
-      <c r="I21" s="9" t="inlineStr"/>
+          <t>2026/05/20</t>
+        </is>
+      </c>
+      <c r="I21" s="9" t="inlineStr">
+        <is>
+          <t>2026/06/27</t>
+        </is>
+      </c>
       <c r="J21" s="9" t="inlineStr"/>
       <c r="K21" s="9" t="inlineStr">
         <is>
@@ -2125,7 +2121,7 @@
       </c>
       <c r="O21" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX Next + DDR5: follow RPL HX Refresh, 待RPL HX Next QS sample WW49到料後安排MVT</t>
+          <t>RPL-HX Next+ DDR4: follow RPL HX Refresh, 待RPL HX Next QS sample WW49到料後安排MVT</t>
         </is>
       </c>
       <c r="P21" s="11" t="inlineStr">
@@ -2145,7 +2141,7 @@
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>Katana 18 HX A2WGXOK</t>
+          <t>Katana 18 HX A2WGXK</t>
         </is>
       </c>
       <c r="D22" s="12" t="inlineStr">
@@ -2170,14 +2166,10 @@
       </c>
       <c r="H22" s="9" t="inlineStr">
         <is>
-          <t>2026/05/20</t>
-        </is>
-      </c>
-      <c r="I22" s="9" t="inlineStr">
-        <is>
-          <t>2026/06/27</t>
-        </is>
-      </c>
+          <t>2026/05/08</t>
+        </is>
+      </c>
+      <c r="I22" s="9" t="inlineStr"/>
       <c r="J22" s="9" t="inlineStr"/>
       <c r="K22" s="9" t="inlineStr">
         <is>
@@ -2201,154 +2193,158 @@
       </c>
       <c r="O22" s="11" t="inlineStr">
         <is>
+          <t>RPL-HX Next + DDR5: follow RPL HX Refresh, 待RPL HX Next QS sample WW49到料後安排MVT</t>
+        </is>
+      </c>
+      <c r="P22" s="11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" hidden="1" outlineLevel="1">
+      <c r="A23" s="7" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>1861</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>Katana 18 HX A2WGXOK</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>RPL-HX Next 55W</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>RTX 5070</t>
+        </is>
+      </c>
+      <c r="G23" s="9" t="inlineStr">
+        <is>
+          <t>顧曉琴</t>
+        </is>
+      </c>
+      <c r="H23" s="9" t="inlineStr">
+        <is>
+          <t>2026/05/20</t>
+        </is>
+      </c>
+      <c r="I23" s="9" t="inlineStr">
+        <is>
+          <t>2026/06/27</t>
+        </is>
+      </c>
+      <c r="J23" s="9" t="inlineStr"/>
+      <c r="K23" s="9" t="inlineStr">
+        <is>
+          <t>2026/12/08</t>
+        </is>
+      </c>
+      <c r="L23" s="9" t="inlineStr">
+        <is>
+          <t>2026/12/30</t>
+        </is>
+      </c>
+      <c r="M23" s="9" t="inlineStr">
+        <is>
+          <t>2027/01/19</t>
+        </is>
+      </c>
+      <c r="N23" s="9" t="inlineStr">
+        <is>
+          <t>2027/01/30</t>
+        </is>
+      </c>
+      <c r="O23" s="11" t="inlineStr">
+        <is>
           <t>RPL-HX Next+ DDR4: follow RPL HX Refresh, 待RPL HX Next QS sample WW49到料後安排MVT</t>
         </is>
       </c>
-      <c r="P22" s="11" t="inlineStr">
+      <c r="P23" s="11" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>265L</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>Crosshair A16 HX E9WEK</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr">
         <is>
           <t>MVT</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="E24" s="4" t="inlineStr">
         <is>
           <t>FRG-HX3D 55W</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr">
+      <c r="F24" s="4" t="inlineStr">
         <is>
           <t>RTX 5050</t>
         </is>
       </c>
-      <c r="G23" s="4" t="inlineStr">
+      <c r="G24" s="4" t="inlineStr">
         <is>
           <t>朱欣怡</t>
         </is>
       </c>
-      <c r="H23" s="4" t="inlineStr">
+      <c r="H24" s="4" t="inlineStr">
         <is>
           <t>2025/10/22</t>
         </is>
       </c>
-      <c r="I23" s="4" t="inlineStr"/>
-      <c r="J23" s="4" t="inlineStr"/>
-      <c r="K23" s="4" t="inlineStr">
+      <c r="I24" s="4" t="inlineStr"/>
+      <c r="J24" s="4" t="inlineStr"/>
+      <c r="K24" s="4" t="inlineStr">
         <is>
           <t>2026/09/21</t>
         </is>
       </c>
-      <c r="L23" s="4" t="inlineStr">
+      <c r="L24" s="4" t="inlineStr">
         <is>
           <t>2026/11/09</t>
         </is>
       </c>
-      <c r="M23" s="4" t="inlineStr">
+      <c r="M24" s="4" t="inlineStr">
         <is>
           <t>2026/12/06</t>
         </is>
       </c>
-      <c r="N23" s="4" t="inlineStr">
+      <c r="N24" s="4" t="inlineStr">
         <is>
           <t>2026/12/16</t>
         </is>
       </c>
-      <c r="O23" s="6" t="inlineStr">
+      <c r="O24" s="6" t="inlineStr">
         <is>
           <t>8/19 Resume並新增new CPU R7 9800HX3D驗證, MVT SMT@9/20</t>
         </is>
       </c>
-      <c r="P23" s="6" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" hidden="1" outlineLevel="1">
-      <c r="A24" s="7" t="n">
-        <v>23</v>
-      </c>
-      <c r="B24" s="8" t="inlineStr">
-        <is>
-          <t>265L</t>
-        </is>
-      </c>
-      <c r="C24" s="9" t="inlineStr">
-        <is>
-          <t>Crosshair A16 HX E9WFK</t>
-        </is>
-      </c>
-      <c r="D24" s="10" t="inlineStr">
-        <is>
-          <t>MVT</t>
-        </is>
-      </c>
-      <c r="E24" s="9" t="inlineStr">
-        <is>
-          <t>FRG-HX3D 55W</t>
-        </is>
-      </c>
-      <c r="F24" s="9" t="inlineStr">
-        <is>
-          <t>RTX 5060</t>
-        </is>
-      </c>
-      <c r="G24" s="9" t="inlineStr">
-        <is>
-          <t>朱欣怡</t>
-        </is>
-      </c>
-      <c r="H24" s="9" t="inlineStr">
-        <is>
-          <t>2025/10/22</t>
-        </is>
-      </c>
-      <c r="I24" s="9" t="inlineStr"/>
-      <c r="J24" s="9" t="inlineStr"/>
-      <c r="K24" s="9" t="inlineStr">
-        <is>
-          <t>2026/09/21</t>
-        </is>
-      </c>
-      <c r="L24" s="9" t="inlineStr">
-        <is>
-          <t>2026/11/09</t>
-        </is>
-      </c>
-      <c r="M24" s="9" t="inlineStr">
-        <is>
-          <t>2026/12/06</t>
-        </is>
-      </c>
-      <c r="N24" s="9" t="inlineStr">
-        <is>
-          <t>2026/12/16</t>
-        </is>
-      </c>
-      <c r="O24" s="11" t="inlineStr">
-        <is>
-          <t>8/19 Resume並新增new CPU R7 9800HX3D</t>
-        </is>
-      </c>
-      <c r="P24" s="11" t="inlineStr">
+      <c r="P24" s="6" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -2365,7 +2361,7 @@
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>Crosshair A16 HX E9WGK</t>
+          <t>Crosshair A16 HX E9WFK</t>
         </is>
       </c>
       <c r="D25" s="10" t="inlineStr">
@@ -2380,7 +2376,7 @@
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t>RTX 5070</t>
+          <t>RTX 5060</t>
         </is>
       </c>
       <c r="G25" s="9" t="inlineStr">
@@ -2437,7 +2433,7 @@
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>Crosshair A16 HX E9WGXK</t>
+          <t>Crosshair A16 HX E9WGK</t>
         </is>
       </c>
       <c r="D26" s="10" t="inlineStr">
@@ -2498,164 +2494,157 @@
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="2" t="n">
+    <row r="27" hidden="1" outlineLevel="1">
+      <c r="A27" s="7" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>2633</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>Stealth 16 AI+ B4WI</t>
-        </is>
-      </c>
-      <c r="D27" s="13" t="inlineStr">
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>265L</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t>Crosshair A16 HX E9WGXK</t>
+        </is>
+      </c>
+      <c r="D27" s="10" t="inlineStr">
+        <is>
+          <t>MVT</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="inlineStr">
+        <is>
+          <t>FRG-HX3D 55W</t>
+        </is>
+      </c>
+      <c r="F27" s="9" t="inlineStr">
+        <is>
+          <t>RTX 5070</t>
+        </is>
+      </c>
+      <c r="G27" s="9" t="inlineStr">
+        <is>
+          <t>朱欣怡</t>
+        </is>
+      </c>
+      <c r="H27" s="9" t="inlineStr">
+        <is>
+          <t>2025/10/22</t>
+        </is>
+      </c>
+      <c r="I27" s="9" t="inlineStr"/>
+      <c r="J27" s="9" t="inlineStr"/>
+      <c r="K27" s="9" t="inlineStr">
+        <is>
+          <t>2026/09/21</t>
+        </is>
+      </c>
+      <c r="L27" s="9" t="inlineStr">
+        <is>
+          <t>2026/11/09</t>
+        </is>
+      </c>
+      <c r="M27" s="9" t="inlineStr">
+        <is>
+          <t>2026/12/06</t>
+        </is>
+      </c>
+      <c r="N27" s="9" t="inlineStr">
+        <is>
+          <t>2026/12/16</t>
+        </is>
+      </c>
+      <c r="O27" s="11" t="inlineStr">
+        <is>
+          <t>8/19 Resume並新增new CPU R7 9800HX3D</t>
+        </is>
+      </c>
+      <c r="P27" s="11" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>2634</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Stealth 16 AI+ B4WE</t>
+        </is>
+      </c>
+      <c r="D28" s="13" t="inlineStr">
         <is>
           <t>EVT</t>
         </is>
       </c>
-      <c r="E27" s="4" t="inlineStr">
+      <c r="E28" s="4" t="inlineStr">
         <is>
           <t>NVL-H 45W</t>
         </is>
       </c>
-      <c r="F27" s="4" t="inlineStr">
-        <is>
-          <t>RTX 5080</t>
-        </is>
-      </c>
-      <c r="G27" s="4" t="inlineStr">
-        <is>
-          <t>朱欣怡</t>
-        </is>
-      </c>
-      <c r="H27" s="4" t="inlineStr">
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>RTX 5050</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>賴雪鳳</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
         <is>
           <t>2026/05/22</t>
         </is>
       </c>
-      <c r="I27" s="4" t="inlineStr">
-        <is>
-          <t>2026/07/23</t>
-        </is>
-      </c>
-      <c r="J27" s="4" t="inlineStr">
-        <is>
-          <t>2026/09/16</t>
-        </is>
-      </c>
-      <c r="K27" s="4" t="inlineStr">
+      <c r="I28" s="4" t="inlineStr">
+        <is>
+          <t>2026/07/31</t>
+        </is>
+      </c>
+      <c r="J28" s="4" t="inlineStr">
+        <is>
+          <t>2026/09/17</t>
+        </is>
+      </c>
+      <c r="K28" s="4" t="inlineStr">
         <is>
           <t>2026/11/11</t>
         </is>
       </c>
-      <c r="L27" s="4" t="inlineStr">
-        <is>
-          <t>2026/11/30</t>
-        </is>
-      </c>
-      <c r="M27" s="4" t="inlineStr">
+      <c r="L28" s="4" t="inlineStr">
+        <is>
+          <t>2026/11/27</t>
+        </is>
+      </c>
+      <c r="M28" s="4" t="inlineStr">
         <is>
           <t>2026/12/29</t>
         </is>
       </c>
-      <c r="N27" s="4" t="inlineStr">
+      <c r="N28" s="4" t="inlineStr">
         <is>
           <t>2027/01/11</t>
         </is>
       </c>
-      <c r="O27" s="6" t="inlineStr">
-        <is>
-          <t>DQA 測試中</t>
-        </is>
-      </c>
-      <c r="P27" s="6" t="inlineStr">
-        <is>
-          <t>1)S1J-AE6C002-TH1 Panel 在 NVL-H平台 無法調亮度,已經請Intel 協助;
-2) Schedule:NV VBIOS @1/6, gating 8天,預計12/E 拿到WHQL，可能影響到最終TTM 時間</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" hidden="1" outlineLevel="1">
-      <c r="A28" s="7" t="n">
-        <v>27</v>
-      </c>
-      <c r="B28" s="8" t="inlineStr">
-        <is>
-          <t>2633</t>
-        </is>
-      </c>
-      <c r="C28" s="9" t="inlineStr">
-        <is>
-          <t>Stealth 16 AI+ B4WH</t>
-        </is>
-      </c>
-      <c r="D28" s="14" t="inlineStr">
-        <is>
-          <t>EVT</t>
-        </is>
-      </c>
-      <c r="E28" s="9" t="inlineStr">
-        <is>
-          <t>NVL-H 45W</t>
-        </is>
-      </c>
-      <c r="F28" s="9" t="inlineStr">
-        <is>
-          <t>RTX 5070Ti</t>
-        </is>
-      </c>
-      <c r="G28" s="9" t="inlineStr">
-        <is>
-          <t>朱欣怡</t>
-        </is>
-      </c>
-      <c r="H28" s="9" t="inlineStr">
-        <is>
-          <t>2026/05/22</t>
-        </is>
-      </c>
-      <c r="I28" s="9" t="inlineStr">
-        <is>
-          <t>2026/07/23</t>
-        </is>
-      </c>
-      <c r="J28" s="9" t="inlineStr">
-        <is>
-          <t>2026/09/16</t>
-        </is>
-      </c>
-      <c r="K28" s="9" t="inlineStr">
-        <is>
-          <t>2026/11/11</t>
-        </is>
-      </c>
-      <c r="L28" s="9" t="inlineStr">
-        <is>
-          <t>2026/11/30</t>
-        </is>
-      </c>
-      <c r="M28" s="9" t="inlineStr">
-        <is>
-          <t>2026/12/29</t>
-        </is>
-      </c>
-      <c r="N28" s="9" t="inlineStr">
-        <is>
-          <t>2027/01/11</t>
-        </is>
-      </c>
-      <c r="O28" s="11" t="inlineStr">
-        <is>
-          <t>DQA 測試中</t>
-        </is>
-      </c>
-      <c r="P28" s="11" t="inlineStr">
-        <is>
-          <t>NA</t>
+      <c r="O28" s="6" t="inlineStr">
+        <is>
+          <t>EVT驗證: PCBA 於9/21調撥回台,機台9/24先發給DQA驗證,其餘節後調撥回台</t>
+        </is>
+      </c>
+      <c r="P28" s="6" t="inlineStr">
+        <is>
+          <t>1)NV VBIOS 驗證時間6周
+2)Intel WHQL :12/E 拿到 可能影響到最終TTM 時間
+3)備料: OLED panel 因無法調亮度問題目前還在找對策,可能影響出貨</t>
         </is>
       </c>
     </row>
@@ -2665,12 +2654,12 @@
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>2633</t>
+          <t>2634</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>Stealth 16 AI+ B4WJ</t>
+          <t>Stealth 16 AI+ B4WF</t>
         </is>
       </c>
       <c r="D29" s="14" t="inlineStr">
@@ -2685,12 +2674,12 @@
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>RTX 5090</t>
+          <t>RTX 5060</t>
         </is>
       </c>
       <c r="G29" s="9" t="inlineStr">
         <is>
-          <t>朱欣怡</t>
+          <t>賴雪鳳</t>
         </is>
       </c>
       <c r="H29" s="9" t="inlineStr">
@@ -2700,12 +2689,12 @@
       </c>
       <c r="I29" s="9" t="inlineStr">
         <is>
-          <t>2026/07/23</t>
+          <t>2026/07/31</t>
         </is>
       </c>
       <c r="J29" s="9" t="inlineStr">
         <is>
-          <t>2026/09/16</t>
+          <t>2026/09/17</t>
         </is>
       </c>
       <c r="K29" s="9" t="inlineStr">
@@ -2715,7 +2704,7 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>2026/11/30</t>
+          <t>2026/11/27</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
@@ -2730,90 +2719,10 @@
       </c>
       <c r="O29" s="11" t="inlineStr">
         <is>
-          <t>DQA 測試中</t>
+          <t>EVT驗證: PCBA 於9/21調撥回台,機台9/24先發給DQA驗證,其餘節後調撥回台</t>
         </is>
       </c>
       <c r="P29" s="11" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="n">
-        <v>29</v>
-      </c>
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>2634</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>Stealth 16 AI+ B4WE</t>
-        </is>
-      </c>
-      <c r="D30" s="13" t="inlineStr">
-        <is>
-          <t>EVT</t>
-        </is>
-      </c>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t>NVL-H 45W</t>
-        </is>
-      </c>
-      <c r="F30" s="4" t="inlineStr">
-        <is>
-          <t>RTX 5050</t>
-        </is>
-      </c>
-      <c r="G30" s="4" t="inlineStr">
-        <is>
-          <t>賴雪鳳</t>
-        </is>
-      </c>
-      <c r="H30" s="4" t="inlineStr">
-        <is>
-          <t>2026/05/22</t>
-        </is>
-      </c>
-      <c r="I30" s="4" t="inlineStr">
-        <is>
-          <t>2026/07/31</t>
-        </is>
-      </c>
-      <c r="J30" s="4" t="inlineStr">
-        <is>
-          <t>2026/09/17</t>
-        </is>
-      </c>
-      <c r="K30" s="4" t="inlineStr">
-        <is>
-          <t>2026/11/11</t>
-        </is>
-      </c>
-      <c r="L30" s="4" t="inlineStr">
-        <is>
-          <t>2026/11/27</t>
-        </is>
-      </c>
-      <c r="M30" s="4" t="inlineStr">
-        <is>
-          <t>2026/12/29</t>
-        </is>
-      </c>
-      <c r="N30" s="4" t="inlineStr">
-        <is>
-          <t>2027/01/11</t>
-        </is>
-      </c>
-      <c r="O30" s="6" t="inlineStr">
-        <is>
-          <t>EVT驗證: PCBA 於9/21調撥回台,機台9/24先發給DQA驗證,其餘節後調撥回台</t>
-        </is>
-      </c>
-      <c r="P30" s="6" t="inlineStr">
         <is>
           <t>1)NV VBIOS 驗證時間6周
 2)Intel WHQL :12/E 拿到 可能影響到最終TTM 時間
@@ -2821,6 +2730,88 @@
         </is>
       </c>
     </row>
+    <row r="30" hidden="1" outlineLevel="1">
+      <c r="A30" s="7" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>2634</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>Stealth 16 AI+ B4WG/GD7 8GB</t>
+        </is>
+      </c>
+      <c r="D30" s="14" t="inlineStr">
+        <is>
+          <t>EVT</t>
+        </is>
+      </c>
+      <c r="E30" s="9" t="inlineStr">
+        <is>
+          <t>NVL-H 45W</t>
+        </is>
+      </c>
+      <c r="F30" s="9" t="inlineStr">
+        <is>
+          <t>RTX 5070</t>
+        </is>
+      </c>
+      <c r="G30" s="9" t="inlineStr">
+        <is>
+          <t>賴雪鳳</t>
+        </is>
+      </c>
+      <c r="H30" s="9" t="inlineStr">
+        <is>
+          <t>2026/05/22</t>
+        </is>
+      </c>
+      <c r="I30" s="9" t="inlineStr">
+        <is>
+          <t>2026/07/31</t>
+        </is>
+      </c>
+      <c r="J30" s="9" t="inlineStr">
+        <is>
+          <t>2026/09/17</t>
+        </is>
+      </c>
+      <c r="K30" s="9" t="inlineStr">
+        <is>
+          <t>2026/11/11</t>
+        </is>
+      </c>
+      <c r="L30" s="9" t="inlineStr">
+        <is>
+          <t>2026/11/27</t>
+        </is>
+      </c>
+      <c r="M30" s="9" t="inlineStr">
+        <is>
+          <t>2026/12/29</t>
+        </is>
+      </c>
+      <c r="N30" s="9" t="inlineStr">
+        <is>
+          <t>2027/01/11</t>
+        </is>
+      </c>
+      <c r="O30" s="11" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P30" s="11" t="inlineStr">
+        <is>
+          <t>1)NV VBIOS 驗證時間6周
+2)Intel WHQL :12/E 拿到 可能影響到最終TTM 時間
+3)備料: OLED panel 因無法調亮度問題目前還在找對策,可能影響出貨</t>
+        </is>
+      </c>
+    </row>
     <row r="31" hidden="1" outlineLevel="1">
       <c r="A31" s="7" t="n">
         <v>30</v>
@@ -2832,7 +2823,7 @@
       </c>
       <c r="C31" s="9" t="inlineStr">
         <is>
-          <t>Stealth 16 AI+ B4WF</t>
+          <t>Stealth 16 AI+ B4WGX/GD7 12GB</t>
         </is>
       </c>
       <c r="D31" s="14" t="inlineStr">
@@ -2847,7 +2838,7 @@
       </c>
       <c r="F31" s="9" t="inlineStr">
         <is>
-          <t>RTX 5060</t>
+          <t>RTX 5070</t>
         </is>
       </c>
       <c r="G31" s="9" t="inlineStr">
@@ -2903,167 +2894,163 @@
         </is>
       </c>
     </row>
-    <row r="32" hidden="1" outlineLevel="1">
-      <c r="A32" s="7" t="n">
+    <row r="32">
+      <c r="A32" s="2" t="n">
         <v>31</v>
       </c>
-      <c r="B32" s="8" t="inlineStr">
-        <is>
-          <t>2634</t>
-        </is>
-      </c>
-      <c r="C32" s="9" t="inlineStr">
-        <is>
-          <t>Stealth 16 AI+ B4WG/GD7 8GB</t>
-        </is>
-      </c>
-      <c r="D32" s="14" t="inlineStr">
-        <is>
-          <t>EVT</t>
-        </is>
-      </c>
-      <c r="E32" s="9" t="inlineStr">
-        <is>
-          <t>NVL-H 45W</t>
-        </is>
-      </c>
-      <c r="F32" s="9" t="inlineStr">
-        <is>
-          <t>RTX 5070</t>
-        </is>
-      </c>
-      <c r="G32" s="9" t="inlineStr">
-        <is>
-          <t>賴雪鳳</t>
-        </is>
-      </c>
-      <c r="H32" s="9" t="inlineStr">
-        <is>
-          <t>2026/05/22</t>
-        </is>
-      </c>
-      <c r="I32" s="9" t="inlineStr">
-        <is>
-          <t>2026/07/31</t>
-        </is>
-      </c>
-      <c r="J32" s="9" t="inlineStr">
-        <is>
-          <t>2026/09/17</t>
-        </is>
-      </c>
-      <c r="K32" s="9" t="inlineStr">
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>14W1</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Modern 14S H3M</t>
+        </is>
+      </c>
+      <c r="D32" s="15" t="inlineStr">
+        <is>
+          <t>DVT</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>WCL 25W</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>Intel® graphics</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>許婕</t>
+        </is>
+      </c>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>2026/08/11</t>
+        </is>
+      </c>
+      <c r="I32" s="4" t="inlineStr">
+        <is>
+          <t>2026/09/23</t>
+        </is>
+      </c>
+      <c r="J32" s="4" t="inlineStr">
         <is>
           <t>2026/11/11</t>
         </is>
       </c>
-      <c r="L32" s="9" t="inlineStr">
-        <is>
-          <t>2026/11/27</t>
-        </is>
-      </c>
-      <c r="M32" s="9" t="inlineStr">
-        <is>
-          <t>2026/12/29</t>
-        </is>
-      </c>
-      <c r="N32" s="9" t="inlineStr">
-        <is>
-          <t>2027/01/11</t>
-        </is>
-      </c>
-      <c r="O32" s="11" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="P32" s="11" t="inlineStr">
-        <is>
-          <t>1)NV VBIOS 驗證時間6周
-2)Intel WHQL :12/E 拿到 可能影響到最終TTM 時間
-3)備料: OLED panel 因無法調亮度問題目前還在找對策,可能影響出貨</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" hidden="1" outlineLevel="1">
-      <c r="A33" s="7" t="n">
+      <c r="K32" s="4" t="inlineStr">
+        <is>
+          <t>2026/12/14</t>
+        </is>
+      </c>
+      <c r="L32" s="4" t="inlineStr">
+        <is>
+          <t>2026/12/18</t>
+        </is>
+      </c>
+      <c r="M32" s="4" t="inlineStr">
+        <is>
+          <t>2027/01/15</t>
+        </is>
+      </c>
+      <c r="N32" s="4" t="inlineStr">
+        <is>
+          <t>2027/01/25</t>
+        </is>
+      </c>
+      <c r="O32" s="6" t="inlineStr">
+        <is>
+          <t>9/23 DVT SMT，已請HW 24號hand carry回台測試</t>
+        </is>
+      </c>
+      <c r="P32" s="6" t="inlineStr">
+        <is>
+          <t>因interposer卡交期delay，0B出圖時間有delay風險，已請power RD與廠商協商採用快掃方式優先確認layout相關測項，10/21確認CPU VRTT 測試結果再來確認0B出圖時間是否調整</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
         <v>32</v>
       </c>
-      <c r="B33" s="8" t="inlineStr">
-        <is>
-          <t>2634</t>
-        </is>
-      </c>
-      <c r="C33" s="9" t="inlineStr">
-        <is>
-          <t>Stealth 16 AI+ B4WGX/GD7 12GB</t>
-        </is>
-      </c>
-      <c r="D33" s="14" t="inlineStr">
-        <is>
-          <t>EVT</t>
-        </is>
-      </c>
-      <c r="E33" s="9" t="inlineStr">
-        <is>
-          <t>NVL-H 45W</t>
-        </is>
-      </c>
-      <c r="F33" s="9" t="inlineStr">
-        <is>
-          <t>RTX 5070</t>
-        </is>
-      </c>
-      <c r="G33" s="9" t="inlineStr">
-        <is>
-          <t>賴雪鳳</t>
-        </is>
-      </c>
-      <c r="H33" s="9" t="inlineStr">
-        <is>
-          <t>2026/05/22</t>
-        </is>
-      </c>
-      <c r="I33" s="9" t="inlineStr">
-        <is>
-          <t>2026/07/31</t>
-        </is>
-      </c>
-      <c r="J33" s="9" t="inlineStr">
-        <is>
-          <t>2026/09/17</t>
-        </is>
-      </c>
-      <c r="K33" s="9" t="inlineStr">
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>2661</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Modern 16S H3M</t>
+        </is>
+      </c>
+      <c r="D33" s="15" t="inlineStr">
+        <is>
+          <t>DVT</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>WCL 25W</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>Intel® graphics</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>許婕</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>2026/08/11</t>
+        </is>
+      </c>
+      <c r="I33" s="4" t="inlineStr">
+        <is>
+          <t>2026/09/23</t>
+        </is>
+      </c>
+      <c r="J33" s="4" t="inlineStr">
         <is>
           <t>2026/11/11</t>
         </is>
       </c>
-      <c r="L33" s="9" t="inlineStr">
-        <is>
-          <t>2026/11/27</t>
-        </is>
-      </c>
-      <c r="M33" s="9" t="inlineStr">
-        <is>
-          <t>2026/12/29</t>
-        </is>
-      </c>
-      <c r="N33" s="9" t="inlineStr">
-        <is>
-          <t>2027/01/11</t>
-        </is>
-      </c>
-      <c r="O33" s="11" t="inlineStr">
-        <is>
-          <t>EVT驗證: PCBA 於9/21調撥回台,機台9/24先發給DQA驗證,其餘節後調撥回台</t>
-        </is>
-      </c>
-      <c r="P33" s="11" t="inlineStr">
-        <is>
-          <t>1)NV VBIOS 驗證時間6周
-2)Intel WHQL :12/E 拿到 可能影響到最終TTM 時間
-3)備料: OLED panel 因無法調亮度問題目前還在找對策,可能影響出貨</t>
+      <c r="K33" s="4" t="inlineStr">
+        <is>
+          <t>2026/12/14</t>
+        </is>
+      </c>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t>2026/12/18</t>
+        </is>
+      </c>
+      <c r="M33" s="4" t="inlineStr">
+        <is>
+          <t>2027/01/15</t>
+        </is>
+      </c>
+      <c r="N33" s="4" t="inlineStr">
+        <is>
+          <t>2027/01/25</t>
+        </is>
+      </c>
+      <c r="O33" s="6" t="inlineStr">
+        <is>
+          <t>9/23 DVT SMT，已請HW 24號hand carry回台測試</t>
+        </is>
+      </c>
+      <c r="P33" s="6" t="inlineStr">
+        <is>
+          <t>因interposer卡交期delay，0B出圖時間有delay風險，已請power RD與廠商協商採用快掃方式優先確認layout相關測項，10/21確認CPU VRTT 測試結果再來確認0B出圖時間是否調整</t>
         </is>
       </c>
     </row>
@@ -3113,32 +3100,32 @@
       </c>
       <c r="J34" s="4" t="inlineStr">
         <is>
-          <t>2026/10/08</t>
+          <t>2026/10/17</t>
         </is>
       </c>
       <c r="K34" s="4" t="inlineStr">
         <is>
-          <t>2026/11/27</t>
+          <t>2026/12/08</t>
         </is>
       </c>
       <c r="L34" s="4" t="inlineStr">
         <is>
-          <t>2026/11/30</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="M34" s="4" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2027/02/16</t>
         </is>
       </c>
       <c r="N34" s="4" t="inlineStr">
         <is>
-          <t>2027/01/11</t>
+          <t>2027/02/26</t>
         </is>
       </c>
       <c r="O34" s="6" t="inlineStr">
         <is>
-          <t>9/10 0B 出圖， EVT SMT：10/8，Pre-Assy：10/9 assy：10/12</t>
+          <t>EVT SMT：10/17，Pre-Assy：10/19 assy：10/21。CPU  W45 delay W48  MVT/ATS Schedule</t>
         </is>
       </c>
       <c r="P34" s="6" t="inlineStr">
@@ -3193,32 +3180,32 @@
       </c>
       <c r="J35" s="9" t="inlineStr">
         <is>
-          <t>2026/10/08</t>
+          <t>2026/10/17</t>
         </is>
       </c>
       <c r="K35" s="9" t="inlineStr">
         <is>
-          <t>2026/11/27</t>
+          <t>2026/12/08</t>
         </is>
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>2026/11/30</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2027/02/16</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>2027/01/11</t>
+          <t>2027/02/26</t>
         </is>
       </c>
       <c r="O35" s="11" t="inlineStr">
         <is>
-          <t>EVT SMT：10/8，Pre-Assy：10/9 assy：10/12</t>
+          <t>EVT SMT：10/17，Pre-Assy：10/19 assy：10/21。CPU  W45 delay W48  MVT/ATS Schedule</t>
         </is>
       </c>
       <c r="P35" s="11" t="inlineStr">
@@ -3269,32 +3256,32 @@
       <c r="I36" s="4" t="inlineStr"/>
       <c r="J36" s="4" t="inlineStr">
         <is>
-          <t>2026/10/08</t>
+          <t>2026/10/17</t>
         </is>
       </c>
       <c r="K36" s="4" t="inlineStr">
         <is>
-          <t>2026/11/27</t>
+          <t>2026/12/08</t>
         </is>
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>2026/11/30</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2027/02/16</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>2027/01/11</t>
+          <t>2027/02/26</t>
         </is>
       </c>
       <c r="O36" s="6" t="inlineStr">
         <is>
-          <t>EVT SMT：10/8，Pre-Assy：10/9 assy：10/12</t>
+          <t>EVT SMT：10/17，Pre-Assy：10/19 assy：10/21。CPU  W45 delay W48  MVT/ATS Schedule</t>
         </is>
       </c>
       <c r="P36" s="6" t="inlineStr">
@@ -3345,32 +3332,32 @@
       <c r="I37" s="9" t="inlineStr"/>
       <c r="J37" s="9" t="inlineStr">
         <is>
-          <t>2026/10/08</t>
+          <t>2026/10/17</t>
         </is>
       </c>
       <c r="K37" s="9" t="inlineStr">
         <is>
-          <t>2026/11/27</t>
+          <t>2026/12/08</t>
         </is>
       </c>
       <c r="L37" s="9" t="inlineStr">
         <is>
-          <t>2026/11/30</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="M37" s="9" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2027/02/16</t>
         </is>
       </c>
       <c r="N37" s="9" t="inlineStr">
         <is>
-          <t>2027/01/11</t>
+          <t>2027/02/26</t>
         </is>
       </c>
       <c r="O37" s="11" t="inlineStr">
         <is>
-          <t>EVT SMT：10/8，Pre-Assy：10/9 assy：10/12</t>
+          <t>EVT SMT：10/17，Pre-Assy：10/19 assy：10/21。CPU  W45 delay W48  MVT/ATS Schedule</t>
         </is>
       </c>
       <c r="P37" s="11" t="inlineStr">
@@ -3385,22 +3372,22 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>13Q5</t>
+          <t>14W2</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Prestige 13 AI+ A4M</t>
-        </is>
-      </c>
-      <c r="D38" s="13" t="inlineStr">
-        <is>
-          <t>EVT</t>
+          <t>Prestige 14S E4M</t>
+        </is>
+      </c>
+      <c r="D38" s="16" t="inlineStr">
+        <is>
+          <t>Design</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>NVL-H 28W</t>
+          <t>NVL-H 30W</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
@@ -3410,56 +3397,50 @@
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>顏春梅</t>
+          <t>吳美芳</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>2026/06/29</t>
+          <t>2026/09/11</t>
         </is>
       </c>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>2026/08/18</t>
+          <t>2026/11/04</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
         <is>
-          <t>2026/10/10</t>
+          <t>2026/12/13</t>
         </is>
       </c>
       <c r="K38" s="4" t="inlineStr">
         <is>
-          <t>2026/11/23</t>
+          <t>2027/01/14</t>
         </is>
       </c>
       <c r="L38" s="4" t="inlineStr">
         <is>
-          <t>2026/12/01</t>
+          <t>2027/01/21</t>
         </is>
       </c>
       <c r="M38" s="4" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2027/02/18</t>
         </is>
       </c>
       <c r="N38" s="4" t="inlineStr">
         <is>
-          <t>2027/01/13</t>
+          <t>2027/02/28</t>
         </is>
       </c>
       <c r="O38" s="6" t="inlineStr">
         <is>
-          <t>EVT 0B SMT@10/10 if 0B fail 0N SMT@11/M</t>
-        </is>
-      </c>
-      <c r="P38" s="6" t="inlineStr">
-        <is>
-          <t>1）schedule: EVT SMT dealy 2天（工廠排程要求物料9/28齊料，PCB 需10/7才能到料）；
-2）備料 PCB 150D 基材10/15 確認，if fail 170Dc 基材11/M PCB才會到料for 測試；
-3）GRL TBT sign FW gap 2W；</t>
-        </is>
-      </c>
+          <t>0A layout中，预计10/26出图</t>
+        </is>
+      </c>
+      <c r="P38" s="6" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -3467,77 +3448,77 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>14W1</t>
+          <t>2662</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Modern 14S H3M</t>
-        </is>
-      </c>
-      <c r="D39" s="15" t="inlineStr">
-        <is>
-          <t>DVT</t>
+          <t>Prestige 16S D4M</t>
+        </is>
+      </c>
+      <c r="D39" s="16" t="inlineStr">
+        <is>
+          <t>Design</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>WCL 25W</t>
+          <t>NVL-H 30W</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>Intel® graphics</t>
+          <t>Intel® Arc™ Graphics</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>許婕</t>
+          <t>吳美芳</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>2026/08/11</t>
+          <t>2026/09/11</t>
         </is>
       </c>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>2026/09/23</t>
+          <t>2026/11/04</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
         <is>
-          <t>2026/11/10</t>
+          <t>2026/12/13</t>
         </is>
       </c>
       <c r="K39" s="4" t="inlineStr">
         <is>
-          <t>2026/12/10</t>
+          <t>2027/01/14</t>
         </is>
       </c>
       <c r="L39" s="4" t="inlineStr">
         <is>
-          <t>2026/12/15</t>
+          <t>2027/01/21</t>
         </is>
       </c>
       <c r="M39" s="4" t="inlineStr">
         <is>
-          <t>2027/01/12</t>
+          <t>2027/02/18</t>
         </is>
       </c>
       <c r="N39" s="4" t="inlineStr">
         <is>
-          <t>2027/01/22</t>
+          <t>2027/02/28</t>
         </is>
       </c>
       <c r="O39" s="6" t="inlineStr">
         <is>
-          <t>9/23 DVT SMT，已請HW 24號hand carry回台測試</t>
+          <t>0A layout中，预计10/26出图</t>
         </is>
       </c>
       <c r="P39" s="6" t="inlineStr">
         <is>
-          <t>改用CSOT FHD 120Hz panel ，ME件交料delay3天，EVT1 pre -Assy与Assy顺延，请ME帮忙pull in EVT2厂商交料，后续schedule暂时保持不变</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -3547,72 +3528,72 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>2661</t>
+          <t>2633</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Modern 16S H3M</t>
-        </is>
-      </c>
-      <c r="D40" s="15" t="inlineStr">
-        <is>
-          <t>DVT</t>
+          <t>Stealth 16 AI+ B4WH</t>
+        </is>
+      </c>
+      <c r="D40" s="13" t="inlineStr">
+        <is>
+          <t>EVT</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>WCL 25W</t>
+          <t>NVL-H 45W</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>Intel® graphics</t>
+          <t>RTX 5070Ti</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>許婕</t>
+          <t>朱欣怡</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>2026/08/11</t>
+          <t>2026/05/22</t>
         </is>
       </c>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>2026/09/23</t>
+          <t>2026/07/23</t>
         </is>
       </c>
       <c r="J40" s="4" t="inlineStr">
         <is>
-          <t>2026/11/10</t>
+          <t>2026/09/16</t>
         </is>
       </c>
       <c r="K40" s="4" t="inlineStr">
         <is>
-          <t>2026/12/10</t>
+          <t>2026/12/02</t>
         </is>
       </c>
       <c r="L40" s="4" t="inlineStr">
         <is>
-          <t>2026/12/15</t>
+          <t>2027/01/13</t>
         </is>
       </c>
       <c r="M40" s="4" t="inlineStr">
         <is>
-          <t>2027/01/12</t>
+          <t>2027/02/23</t>
         </is>
       </c>
       <c r="N40" s="4" t="inlineStr">
         <is>
-          <t>2027/01/22</t>
+          <t>2027/03/05</t>
         </is>
       </c>
       <c r="O40" s="6" t="inlineStr">
         <is>
-          <t>9/23 DVT SMT，已請HW 24號hand carry回台測試</t>
+          <t>DQA 測試中</t>
         </is>
       </c>
       <c r="P40" s="6" t="inlineStr">
@@ -3621,157 +3602,161 @@
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="2" t="n">
+    <row r="41" hidden="1" outlineLevel="1">
+      <c r="A41" s="7" t="n">
         <v>40</v>
       </c>
-      <c r="B41" s="3" t="inlineStr">
-        <is>
-          <t>14W2</t>
-        </is>
-      </c>
-      <c r="C41" s="4" t="inlineStr">
-        <is>
-          <t>Prestige 14S E4M</t>
-        </is>
-      </c>
-      <c r="D41" s="16" t="inlineStr">
-        <is>
-          <t>Design</t>
-        </is>
-      </c>
-      <c r="E41" s="4" t="inlineStr">
-        <is>
-          <t>NVL-H 30W</t>
-        </is>
-      </c>
-      <c r="F41" s="4" t="inlineStr">
-        <is>
-          <t>Intel® Arc™ Graphics</t>
-        </is>
-      </c>
-      <c r="G41" s="4" t="inlineStr">
-        <is>
-          <t>吳美芳</t>
-        </is>
-      </c>
-      <c r="H41" s="4" t="inlineStr">
-        <is>
-          <t>2026/09/11</t>
-        </is>
-      </c>
-      <c r="I41" s="4" t="inlineStr">
-        <is>
-          <t>2026/11/04</t>
-        </is>
-      </c>
-      <c r="J41" s="4" t="inlineStr">
-        <is>
-          <t>2026/12/13</t>
-        </is>
-      </c>
-      <c r="K41" s="4" t="inlineStr">
-        <is>
-          <t>2027/01/14</t>
-        </is>
-      </c>
-      <c r="L41" s="4" t="inlineStr">
-        <is>
-          <t>2027/01/21</t>
-        </is>
-      </c>
-      <c r="M41" s="4" t="inlineStr">
-        <is>
-          <t>2027/02/18</t>
-        </is>
-      </c>
-      <c r="N41" s="4" t="inlineStr">
-        <is>
-          <t>2027/02/28</t>
-        </is>
-      </c>
-      <c r="O41" s="6" t="inlineStr">
-        <is>
-          <t>0A layout中，预计10/26出图</t>
-        </is>
-      </c>
-      <c r="P41" s="6" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="n">
+      <c r="B41" s="8" t="inlineStr">
+        <is>
+          <t>2633</t>
+        </is>
+      </c>
+      <c r="C41" s="9" t="inlineStr">
+        <is>
+          <t>Stealth 16 AI+ B4WI</t>
+        </is>
+      </c>
+      <c r="D41" s="14" t="inlineStr">
+        <is>
+          <t>EVT</t>
+        </is>
+      </c>
+      <c r="E41" s="9" t="inlineStr">
+        <is>
+          <t>NVL-H 45W</t>
+        </is>
+      </c>
+      <c r="F41" s="9" t="inlineStr">
+        <is>
+          <t>RTX 5080</t>
+        </is>
+      </c>
+      <c r="G41" s="9" t="inlineStr">
+        <is>
+          <t>朱欣怡</t>
+        </is>
+      </c>
+      <c r="H41" s="9" t="inlineStr">
+        <is>
+          <t>2026/05/22</t>
+        </is>
+      </c>
+      <c r="I41" s="9" t="inlineStr">
+        <is>
+          <t>2026/07/23</t>
+        </is>
+      </c>
+      <c r="J41" s="9" t="inlineStr">
+        <is>
+          <t>2026/09/16</t>
+        </is>
+      </c>
+      <c r="K41" s="9" t="inlineStr">
+        <is>
+          <t>2026/12/02</t>
+        </is>
+      </c>
+      <c r="L41" s="9" t="inlineStr">
+        <is>
+          <t>2027/01/13</t>
+        </is>
+      </c>
+      <c r="M41" s="9" t="inlineStr">
+        <is>
+          <t>2027/02/23</t>
+        </is>
+      </c>
+      <c r="N41" s="9" t="inlineStr">
+        <is>
+          <t>2027/03/05</t>
+        </is>
+      </c>
+      <c r="O41" s="11" t="inlineStr">
+        <is>
+          <t>DQA 測試中</t>
+        </is>
+      </c>
+      <c r="P41" s="11" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" hidden="1" outlineLevel="1">
+      <c r="A42" s="7" t="n">
         <v>41</v>
       </c>
-      <c r="B42" s="3" t="inlineStr">
-        <is>
-          <t>2662</t>
-        </is>
-      </c>
-      <c r="C42" s="4" t="inlineStr">
-        <is>
-          <t>Prestige 16S D4M</t>
-        </is>
-      </c>
-      <c r="D42" s="16" t="inlineStr">
-        <is>
-          <t>Design</t>
-        </is>
-      </c>
-      <c r="E42" s="4" t="inlineStr">
-        <is>
-          <t>NVL-H 30W</t>
-        </is>
-      </c>
-      <c r="F42" s="4" t="inlineStr">
-        <is>
-          <t>Intel® Arc™ Graphics</t>
-        </is>
-      </c>
-      <c r="G42" s="4" t="inlineStr">
-        <is>
-          <t>吳美芳</t>
-        </is>
-      </c>
-      <c r="H42" s="4" t="inlineStr">
-        <is>
-          <t>2026/09/11</t>
-        </is>
-      </c>
-      <c r="I42" s="4" t="inlineStr">
-        <is>
-          <t>2026/11/04</t>
-        </is>
-      </c>
-      <c r="J42" s="4" t="inlineStr">
-        <is>
-          <t>2026/12/13</t>
-        </is>
-      </c>
-      <c r="K42" s="4" t="inlineStr">
-        <is>
-          <t>2027/01/14</t>
-        </is>
-      </c>
-      <c r="L42" s="4" t="inlineStr">
-        <is>
-          <t>2027/01/21</t>
-        </is>
-      </c>
-      <c r="M42" s="4" t="inlineStr">
-        <is>
-          <t>2027/02/18</t>
-        </is>
-      </c>
-      <c r="N42" s="4" t="inlineStr">
-        <is>
-          <t>2027/02/28</t>
-        </is>
-      </c>
-      <c r="O42" s="6" t="inlineStr">
-        <is>
-          <t>0A layout中，预计10/26出图</t>
-        </is>
-      </c>
-      <c r="P42" s="6" t="inlineStr">
+      <c r="B42" s="8" t="inlineStr">
+        <is>
+          <t>2633</t>
+        </is>
+      </c>
+      <c r="C42" s="9" t="inlineStr">
+        <is>
+          <t>Stealth 16 AI+ B4WJ</t>
+        </is>
+      </c>
+      <c r="D42" s="14" t="inlineStr">
+        <is>
+          <t>EVT</t>
+        </is>
+      </c>
+      <c r="E42" s="9" t="inlineStr">
+        <is>
+          <t>NVL-H 45W</t>
+        </is>
+      </c>
+      <c r="F42" s="9" t="inlineStr">
+        <is>
+          <t>RTX 5090</t>
+        </is>
+      </c>
+      <c r="G42" s="9" t="inlineStr">
+        <is>
+          <t>朱欣怡</t>
+        </is>
+      </c>
+      <c r="H42" s="9" t="inlineStr">
+        <is>
+          <t>2026/05/22</t>
+        </is>
+      </c>
+      <c r="I42" s="9" t="inlineStr">
+        <is>
+          <t>2026/07/23</t>
+        </is>
+      </c>
+      <c r="J42" s="9" t="inlineStr">
+        <is>
+          <t>2026/09/16</t>
+        </is>
+      </c>
+      <c r="K42" s="9" t="inlineStr">
+        <is>
+          <t>2026/12/02</t>
+        </is>
+      </c>
+      <c r="L42" s="9" t="inlineStr">
+        <is>
+          <t>2027/01/13</t>
+        </is>
+      </c>
+      <c r="M42" s="9" t="inlineStr">
+        <is>
+          <t>2027/02/23</t>
+        </is>
+      </c>
+      <c r="N42" s="9" t="inlineStr">
+        <is>
+          <t>2027/03/05</t>
+        </is>
+      </c>
+      <c r="O42" s="11" t="inlineStr">
+        <is>
+          <t>DQA 測試中</t>
+        </is>
+      </c>
+      <c r="P42" s="11" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -3783,155 +3768,156 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
+          <t>13Q5</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Prestige 13 AI+ A4M</t>
+        </is>
+      </c>
+      <c r="D43" s="13" t="inlineStr">
+        <is>
+          <t>EVT</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>NVL-H 28W</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>Intel® Arc™ Graphics</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>顏春梅</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="inlineStr">
+        <is>
+          <t>2026/06/29</t>
+        </is>
+      </c>
+      <c r="I43" s="4" t="inlineStr">
+        <is>
+          <t>2026/08/18</t>
+        </is>
+      </c>
+      <c r="J43" s="4" t="inlineStr">
+        <is>
+          <t>2026/10/10</t>
+        </is>
+      </c>
+      <c r="K43" s="4" t="inlineStr">
+        <is>
+          <t>2026/12/03</t>
+        </is>
+      </c>
+      <c r="L43" s="4" t="inlineStr">
+        <is>
+          <t>2027/01/22</t>
+        </is>
+      </c>
+      <c r="M43" s="4" t="inlineStr">
+        <is>
+          <t>2027/02/23</t>
+        </is>
+      </c>
+      <c r="N43" s="4" t="inlineStr">
+        <is>
+          <t>2027/03/05</t>
+        </is>
+      </c>
+      <c r="O43" s="6" t="inlineStr">
+        <is>
+          <t>EVT 0B SMT@10/10 if 0B fail 0N SMT@11/M</t>
+        </is>
+      </c>
+      <c r="P43" s="6" t="inlineStr">
+        <is>
+          <t>1）schedule: intel CPU delay schedule update；
+2）備料 PCB 150D 基材10/15 確認，if fail 170Dc 基材11/M PCB才會到料for 測試；</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
           <t>2654</t>
         </is>
       </c>
-      <c r="C43" s="4" t="inlineStr">
+      <c r="C44" s="4" t="inlineStr">
         <is>
           <t>Raider 16 Max HX B4WH</t>
         </is>
       </c>
-      <c r="D43" s="13" t="inlineStr">
+      <c r="D44" s="13" t="inlineStr">
         <is>
           <t>EVT</t>
         </is>
       </c>
-      <c r="E43" s="4" t="inlineStr">
+      <c r="E44" s="4" t="inlineStr">
         <is>
           <t>NVL-HX 55W</t>
         </is>
       </c>
-      <c r="F43" s="4" t="inlineStr">
+      <c r="F44" s="4" t="inlineStr">
         <is>
           <t>RTX 5070Ti</t>
         </is>
       </c>
-      <c r="G43" s="4" t="inlineStr">
+      <c r="G44" s="4" t="inlineStr">
         <is>
           <t>吳美芳</t>
         </is>
       </c>
-      <c r="H43" s="4" t="inlineStr">
+      <c r="H44" s="4" t="inlineStr">
         <is>
           <t>2026/05/19</t>
         </is>
       </c>
-      <c r="I43" s="4" t="inlineStr">
+      <c r="I44" s="4" t="inlineStr">
         <is>
           <t>2026/08/05</t>
         </is>
       </c>
-      <c r="J43" s="4" t="inlineStr">
+      <c r="J44" s="4" t="inlineStr">
         <is>
           <t>2026/09/27</t>
         </is>
       </c>
-      <c r="K43" s="4" t="inlineStr">
+      <c r="K44" s="4" t="inlineStr">
         <is>
           <t>2027/01/11</t>
         </is>
       </c>
-      <c r="L43" s="4" t="inlineStr">
+      <c r="L44" s="4" t="inlineStr">
         <is>
           <t>2027/02/02</t>
         </is>
       </c>
-      <c r="M43" s="4" t="inlineStr">
+      <c r="M44" s="4" t="inlineStr">
         <is>
           <t>2027/03/08</t>
         </is>
       </c>
-      <c r="N43" s="4" t="inlineStr">
+      <c r="N44" s="4" t="inlineStr">
         <is>
           <t>2027/03/18</t>
         </is>
       </c>
-      <c r="O43" s="6" t="inlineStr">
+      <c r="O44" s="6" t="inlineStr">
         <is>
           <t>安排9/27 EVT打板，28试组，10/12组装</t>
         </is>
       </c>
-      <c r="P43" s="6" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" hidden="1" outlineLevel="1">
-      <c r="A44" s="7" t="n">
-        <v>43</v>
-      </c>
-      <c r="B44" s="8" t="inlineStr">
-        <is>
-          <t>2654</t>
-        </is>
-      </c>
-      <c r="C44" s="9" t="inlineStr">
-        <is>
-          <t>Raider 16 Max HX B4WI</t>
-        </is>
-      </c>
-      <c r="D44" s="14" t="inlineStr">
-        <is>
-          <t>EVT</t>
-        </is>
-      </c>
-      <c r="E44" s="9" t="inlineStr">
-        <is>
-          <t>NVL-HX 55W</t>
-        </is>
-      </c>
-      <c r="F44" s="9" t="inlineStr">
-        <is>
-          <t>RTX 5080</t>
-        </is>
-      </c>
-      <c r="G44" s="9" t="inlineStr">
-        <is>
-          <t>吳美芳</t>
-        </is>
-      </c>
-      <c r="H44" s="9" t="inlineStr">
-        <is>
-          <t>2026/05/19</t>
-        </is>
-      </c>
-      <c r="I44" s="9" t="inlineStr">
-        <is>
-          <t>2026/08/05</t>
-        </is>
-      </c>
-      <c r="J44" s="9" t="inlineStr">
-        <is>
-          <t>2026/09/27</t>
-        </is>
-      </c>
-      <c r="K44" s="9" t="inlineStr">
-        <is>
-          <t>2027/01/11</t>
-        </is>
-      </c>
-      <c r="L44" s="9" t="inlineStr">
-        <is>
-          <t>2027/02/02</t>
-        </is>
-      </c>
-      <c r="M44" s="9" t="inlineStr">
-        <is>
-          <t>2027/03/08</t>
-        </is>
-      </c>
-      <c r="N44" s="9" t="inlineStr">
-        <is>
-          <t>2027/03/18</t>
-        </is>
-      </c>
-      <c r="O44" s="11" t="inlineStr">
-        <is>
-          <t>安排9/27 EVT打板，28试组，10/12组装</t>
-        </is>
-      </c>
-      <c r="P44" s="11" t="inlineStr">
+      <c r="P44" s="6" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -3948,232 +3934,231 @@
       </c>
       <c r="C45" s="9" t="inlineStr">
         <is>
+          <t>Raider 16 Max HX B4WI</t>
+        </is>
+      </c>
+      <c r="D45" s="14" t="inlineStr">
+        <is>
+          <t>EVT</t>
+        </is>
+      </c>
+      <c r="E45" s="9" t="inlineStr">
+        <is>
+          <t>NVL-HX 55W</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="inlineStr">
+        <is>
+          <t>RTX 5080</t>
+        </is>
+      </c>
+      <c r="G45" s="9" t="inlineStr">
+        <is>
+          <t>吳美芳</t>
+        </is>
+      </c>
+      <c r="H45" s="9" t="inlineStr">
+        <is>
+          <t>2026/05/19</t>
+        </is>
+      </c>
+      <c r="I45" s="9" t="inlineStr">
+        <is>
+          <t>2026/08/05</t>
+        </is>
+      </c>
+      <c r="J45" s="9" t="inlineStr">
+        <is>
+          <t>2026/09/27</t>
+        </is>
+      </c>
+      <c r="K45" s="9" t="inlineStr">
+        <is>
+          <t>2027/01/11</t>
+        </is>
+      </c>
+      <c r="L45" s="9" t="inlineStr">
+        <is>
+          <t>2027/02/02</t>
+        </is>
+      </c>
+      <c r="M45" s="9" t="inlineStr">
+        <is>
+          <t>2027/03/08</t>
+        </is>
+      </c>
+      <c r="N45" s="9" t="inlineStr">
+        <is>
+          <t>2027/03/18</t>
+        </is>
+      </c>
+      <c r="O45" s="11" t="inlineStr">
+        <is>
+          <t>安排9/27 EVT打板，28试组，10/12组装</t>
+        </is>
+      </c>
+      <c r="P45" s="11" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" hidden="1" outlineLevel="1">
+      <c r="A46" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="8" t="inlineStr">
+        <is>
+          <t>2654</t>
+        </is>
+      </c>
+      <c r="C46" s="9" t="inlineStr">
+        <is>
           <t>Raider 16 Max HX B4WJ</t>
         </is>
       </c>
-      <c r="D45" s="14" t="inlineStr">
+      <c r="D46" s="14" t="inlineStr">
         <is>
           <t>EVT</t>
         </is>
       </c>
-      <c r="E45" s="9" t="inlineStr">
+      <c r="E46" s="9" t="inlineStr">
         <is>
           <t>NVL-HX 55W</t>
         </is>
       </c>
-      <c r="F45" s="9" t="inlineStr">
+      <c r="F46" s="9" t="inlineStr">
         <is>
           <t>RTX 5090</t>
         </is>
       </c>
-      <c r="G45" s="9" t="inlineStr">
+      <c r="G46" s="9" t="inlineStr">
         <is>
           <t>吳美芳</t>
         </is>
       </c>
-      <c r="H45" s="9" t="inlineStr">
+      <c r="H46" s="9" t="inlineStr">
         <is>
           <t>2026/05/19</t>
         </is>
       </c>
-      <c r="I45" s="9" t="inlineStr">
+      <c r="I46" s="9" t="inlineStr">
         <is>
           <t>2026/08/05</t>
         </is>
       </c>
-      <c r="J45" s="9" t="inlineStr">
+      <c r="J46" s="9" t="inlineStr">
         <is>
           <t>2026/09/27</t>
         </is>
       </c>
-      <c r="K45" s="9" t="inlineStr">
+      <c r="K46" s="9" t="inlineStr">
         <is>
           <t>2027/01/11</t>
         </is>
       </c>
-      <c r="L45" s="9" t="inlineStr">
+      <c r="L46" s="9" t="inlineStr">
         <is>
           <t>2027/02/02</t>
         </is>
       </c>
-      <c r="M45" s="9" t="inlineStr">
+      <c r="M46" s="9" t="inlineStr">
         <is>
           <t>2027/03/08</t>
         </is>
       </c>
-      <c r="N45" s="9" t="inlineStr">
+      <c r="N46" s="9" t="inlineStr">
         <is>
           <t>2027/03/18</t>
         </is>
       </c>
-      <c r="O45" s="11" t="inlineStr">
+      <c r="O46" s="11" t="inlineStr">
         <is>
           <t>安排9/27 EVT打板，28试组，10/12组装</t>
         </is>
       </c>
-      <c r="P45" s="11" t="inlineStr">
+      <c r="P46" s="11" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="B46" s="3" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
         <is>
           <t>1851</t>
         </is>
       </c>
-      <c r="C46" s="4" t="inlineStr">
+      <c r="C47" s="4" t="inlineStr">
         <is>
           <t>Titan 18 HX B4WH</t>
         </is>
       </c>
-      <c r="D46" s="15" t="inlineStr">
+      <c r="D47" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
       </c>
-      <c r="E46" s="4" t="inlineStr">
+      <c r="E47" s="4" t="inlineStr">
         <is>
           <t>NVL-HX 55W</t>
         </is>
       </c>
-      <c r="F46" s="4" t="inlineStr">
+      <c r="F47" s="4" t="inlineStr">
         <is>
           <t>RTX 5070Ti</t>
         </is>
       </c>
-      <c r="G46" s="4" t="inlineStr">
+      <c r="G47" s="4" t="inlineStr">
         <is>
           <t>高宇奇</t>
         </is>
       </c>
-      <c r="H46" s="4" t="inlineStr">
+      <c r="H47" s="4" t="inlineStr">
         <is>
           <t>2026/06/29</t>
         </is>
       </c>
-      <c r="I46" s="4" t="inlineStr">
+      <c r="I47" s="4" t="inlineStr">
         <is>
           <t>2026/08/19</t>
         </is>
       </c>
-      <c r="J46" s="4" t="inlineStr">
+      <c r="J47" s="4" t="inlineStr">
         <is>
           <t>2026/11/03</t>
         </is>
       </c>
-      <c r="K46" s="4" t="inlineStr">
+      <c r="K47" s="4" t="inlineStr">
         <is>
           <t>2027/01/08</t>
         </is>
       </c>
-      <c r="L46" s="4" t="inlineStr">
+      <c r="L47" s="4" t="inlineStr">
         <is>
           <t>2027/02/01</t>
         </is>
       </c>
-      <c r="M46" s="4" t="inlineStr">
+      <c r="M47" s="4" t="inlineStr">
         <is>
           <t>2027/03/08</t>
         </is>
       </c>
-      <c r="N46" s="4" t="inlineStr">
+      <c r="N47" s="4" t="inlineStr">
         <is>
           <t>2027/03/18</t>
         </is>
       </c>
-      <c r="O46" s="6" t="inlineStr">
+      <c r="O47" s="6" t="inlineStr">
         <is>
           <t>1) DVT板子測試中,SA DP2.1無法測試問題已經跟GRL預約10/7讓SA &amp; EE一起過去GRL debug.
 2) 0N layout進行中,預計10/14 gerber out.</t>
         </is>
       </c>
-      <c r="P46" s="6" t="inlineStr">
-        <is>
-          <t>1) 1851 Titan &amp; Raider取消原本 91.8Wh 的規劃，全系列統一採用 99Wh 電池，新開的99Wh電池開模與備料趕不上 1851 EVT，EVT 試產keep採用原本開案規劃的91.8Wh 電池，後續請電池廠商提供手工模樣品for ME RD於 MVT 前進行初步替換驗證.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" hidden="1" outlineLevel="1">
-      <c r="A47" s="7" t="n">
-        <v>46</v>
-      </c>
-      <c r="B47" s="8" t="inlineStr">
-        <is>
-          <t>1851</t>
-        </is>
-      </c>
-      <c r="C47" s="9" t="inlineStr">
-        <is>
-          <t>Titan 18 HX B4WI</t>
-        </is>
-      </c>
-      <c r="D47" s="17" t="inlineStr">
-        <is>
-          <t>DVT</t>
-        </is>
-      </c>
-      <c r="E47" s="9" t="inlineStr">
-        <is>
-          <t>NVL-HX 55W</t>
-        </is>
-      </c>
-      <c r="F47" s="9" t="inlineStr">
-        <is>
-          <t>RTX 5080</t>
-        </is>
-      </c>
-      <c r="G47" s="9" t="inlineStr">
-        <is>
-          <t>高宇奇</t>
-        </is>
-      </c>
-      <c r="H47" s="9" t="inlineStr">
-        <is>
-          <t>2026/06/29</t>
-        </is>
-      </c>
-      <c r="I47" s="9" t="inlineStr">
-        <is>
-          <t>2026/08/19</t>
-        </is>
-      </c>
-      <c r="J47" s="9" t="inlineStr">
-        <is>
-          <t>2026/11/03</t>
-        </is>
-      </c>
-      <c r="K47" s="9" t="inlineStr">
-        <is>
-          <t>2027/01/08</t>
-        </is>
-      </c>
-      <c r="L47" s="9" t="inlineStr">
-        <is>
-          <t>2027/02/01</t>
-        </is>
-      </c>
-      <c r="M47" s="9" t="inlineStr">
-        <is>
-          <t>2027/03/08</t>
-        </is>
-      </c>
-      <c r="N47" s="9" t="inlineStr">
-        <is>
-          <t>2027/03/18</t>
-        </is>
-      </c>
-      <c r="O47" s="11" t="inlineStr">
-        <is>
-          <t>1) DVT板子測試中,SA DP2.1無法測試問題已經跟GRL預約10/7讓SA &amp; EE一起過去GRL debug.
-2) 0N layout進行中,預計10/14 gerber out.</t>
-        </is>
-      </c>
-      <c r="P47" s="11" t="inlineStr">
+      <c r="P47" s="6" t="inlineStr">
         <is>
           <t>1) 1851 Titan &amp; Raider取消原本 91.8Wh 的規劃，全系列統一採用 99Wh 電池，新開的99Wh電池開模與備料趕不上 1851 EVT，EVT 試產keep採用原本開案規劃的91.8Wh 電池，後續請電池廠商提供手工模樣品for ME RD於 MVT 前進行初步替換驗證.</t>
         </is>
@@ -4190,7 +4175,7 @@
       </c>
       <c r="C48" s="9" t="inlineStr">
         <is>
-          <t>Titan 18 HX B4WJ</t>
+          <t>Titan 18 HX B4WI</t>
         </is>
       </c>
       <c r="D48" s="17" t="inlineStr">
@@ -4205,7 +4190,7 @@
       </c>
       <c r="F48" s="9" t="inlineStr">
         <is>
-          <t>RTX 5090</t>
+          <t>RTX 5080</t>
         </is>
       </c>
       <c r="G48" s="9" t="inlineStr">
@@ -4271,7 +4256,7 @@
       </c>
       <c r="C49" s="9" t="inlineStr">
         <is>
-          <t>Raider 18 Max HX B4WH</t>
+          <t>Titan 18 HX B4WJ</t>
         </is>
       </c>
       <c r="D49" s="17" t="inlineStr">
@@ -4286,7 +4271,7 @@
       </c>
       <c r="F49" s="9" t="inlineStr">
         <is>
-          <t>RTX 5070Ti</t>
+          <t>RTX 5090</t>
         </is>
       </c>
       <c r="G49" s="9" t="inlineStr">
@@ -4352,7 +4337,7 @@
       </c>
       <c r="C50" s="9" t="inlineStr">
         <is>
-          <t>Raider 18 Max HX B4WI</t>
+          <t>Raider 18 Max HX B4WH</t>
         </is>
       </c>
       <c r="D50" s="17" t="inlineStr">
@@ -4367,7 +4352,7 @@
       </c>
       <c r="F50" s="9" t="inlineStr">
         <is>
-          <t>RTX 5080</t>
+          <t>RTX 5070Ti</t>
         </is>
       </c>
       <c r="G50" s="9" t="inlineStr">
@@ -4433,7 +4418,7 @@
       </c>
       <c r="C51" s="9" t="inlineStr">
         <is>
-          <t>Raider 18 Max HX B4WJ</t>
+          <t>Raider 18 Max HX B4WI</t>
         </is>
       </c>
       <c r="D51" s="17" t="inlineStr">
@@ -4448,7 +4433,7 @@
       </c>
       <c r="F51" s="9" t="inlineStr">
         <is>
-          <t>RTX 5090</t>
+          <t>RTX 5080</t>
         </is>
       </c>
       <c r="G51" s="9" t="inlineStr">
@@ -4503,161 +4488,162 @@
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="2" t="n">
+    <row r="52" hidden="1" outlineLevel="1">
+      <c r="A52" s="7" t="n">
         <v>51</v>
       </c>
-      <c r="B52" s="3" t="inlineStr">
+      <c r="B52" s="8" t="inlineStr">
+        <is>
+          <t>1851</t>
+        </is>
+      </c>
+      <c r="C52" s="9" t="inlineStr">
+        <is>
+          <t>Raider 18 Max HX B4WJ</t>
+        </is>
+      </c>
+      <c r="D52" s="17" t="inlineStr">
+        <is>
+          <t>DVT</t>
+        </is>
+      </c>
+      <c r="E52" s="9" t="inlineStr">
+        <is>
+          <t>NVL-HX 55W</t>
+        </is>
+      </c>
+      <c r="F52" s="9" t="inlineStr">
+        <is>
+          <t>RTX 5090</t>
+        </is>
+      </c>
+      <c r="G52" s="9" t="inlineStr">
+        <is>
+          <t>高宇奇</t>
+        </is>
+      </c>
+      <c r="H52" s="9" t="inlineStr">
+        <is>
+          <t>2026/06/29</t>
+        </is>
+      </c>
+      <c r="I52" s="9" t="inlineStr">
+        <is>
+          <t>2026/08/19</t>
+        </is>
+      </c>
+      <c r="J52" s="9" t="inlineStr">
+        <is>
+          <t>2026/11/03</t>
+        </is>
+      </c>
+      <c r="K52" s="9" t="inlineStr">
+        <is>
+          <t>2027/01/08</t>
+        </is>
+      </c>
+      <c r="L52" s="9" t="inlineStr">
+        <is>
+          <t>2027/02/01</t>
+        </is>
+      </c>
+      <c r="M52" s="9" t="inlineStr">
+        <is>
+          <t>2027/03/08</t>
+        </is>
+      </c>
+      <c r="N52" s="9" t="inlineStr">
+        <is>
+          <t>2027/03/18</t>
+        </is>
+      </c>
+      <c r="O52" s="11" t="inlineStr">
+        <is>
+          <t>1) DVT板子測試中,SA DP2.1無法測試問題已經跟GRL預約10/7讓SA &amp; EE一起過去GRL debug.
+2) 0N layout進行中,預計10/14 gerber out.</t>
+        </is>
+      </c>
+      <c r="P52" s="11" t="inlineStr">
+        <is>
+          <t>1) 1851 Titan &amp; Raider取消原本 91.8Wh 的規劃，全系列統一採用 99Wh 電池，新開的99Wh電池開模與備料趕不上 1851 EVT，EVT 試產keep採用原本開案規劃的91.8Wh 電池，後續請電池廠商提供手工模樣品for ME RD於 MVT 前進行初步替換驗證.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
         <is>
           <t>2655</t>
         </is>
       </c>
-      <c r="C52" s="4" t="inlineStr">
+      <c r="C53" s="4" t="inlineStr">
         <is>
           <t>Crosshair 16 Max HX E4WEK</t>
         </is>
       </c>
-      <c r="D52" s="13" t="inlineStr">
+      <c r="D53" s="13" t="inlineStr">
         <is>
           <t>EVT</t>
         </is>
       </c>
-      <c r="E52" s="4" t="inlineStr">
+      <c r="E53" s="4" t="inlineStr">
         <is>
           <t>NVL-HX 55W</t>
         </is>
       </c>
-      <c r="F52" s="4" t="inlineStr">
+      <c r="F53" s="4" t="inlineStr">
         <is>
           <t>RTX 5050</t>
         </is>
       </c>
-      <c r="G52" s="4" t="inlineStr">
+      <c r="G53" s="4" t="inlineStr">
         <is>
           <t>鮑佩佩</t>
         </is>
       </c>
-      <c r="H52" s="4" t="inlineStr">
+      <c r="H53" s="4" t="inlineStr">
         <is>
           <t>2026/05/19</t>
         </is>
       </c>
-      <c r="I52" s="4" t="inlineStr">
+      <c r="I53" s="4" t="inlineStr">
         <is>
           <t>2026/08/06</t>
         </is>
       </c>
-      <c r="J52" s="4" t="inlineStr">
+      <c r="J53" s="4" t="inlineStr">
         <is>
           <t>2026/09/27</t>
         </is>
       </c>
-      <c r="K52" s="4" t="inlineStr">
+      <c r="K53" s="4" t="inlineStr">
         <is>
           <t>2027/01/11</t>
         </is>
       </c>
-      <c r="L52" s="4" t="inlineStr">
+      <c r="L53" s="4" t="inlineStr">
         <is>
           <t>2027/02/02</t>
         </is>
       </c>
-      <c r="M52" s="4" t="inlineStr">
+      <c r="M53" s="4" t="inlineStr">
         <is>
           <t>2027/03/08</t>
         </is>
       </c>
-      <c r="N52" s="4" t="inlineStr">
+      <c r="N53" s="4" t="inlineStr">
         <is>
           <t>2027/03/18</t>
         </is>
       </c>
-      <c r="O52" s="6" t="inlineStr">
+      <c r="O53" s="6" t="inlineStr">
         <is>
           <t>9/27 EVT SMT，9/28 Pre Assy，10/9 Assy</t>
         </is>
       </c>
-      <c r="P52" s="6" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" hidden="1" outlineLevel="1">
-      <c r="A53" s="7" t="n">
-        <v>52</v>
-      </c>
-      <c r="B53" s="8" t="inlineStr">
-        <is>
-          <t>2655</t>
-        </is>
-      </c>
-      <c r="C53" s="9" t="inlineStr">
-        <is>
-          <t>Crosshair 16 Max HX E4WFK</t>
-        </is>
-      </c>
-      <c r="D53" s="14" t="inlineStr">
-        <is>
-          <t>EVT</t>
-        </is>
-      </c>
-      <c r="E53" s="9" t="inlineStr">
-        <is>
-          <t>NVL-HX 55W</t>
-        </is>
-      </c>
-      <c r="F53" s="9" t="inlineStr">
-        <is>
-          <t>RTX 5060</t>
-        </is>
-      </c>
-      <c r="G53" s="9" t="inlineStr">
-        <is>
-          <t>鮑佩佩</t>
-        </is>
-      </c>
-      <c r="H53" s="9" t="inlineStr">
-        <is>
-          <t>2026/05/19</t>
-        </is>
-      </c>
-      <c r="I53" s="9" t="inlineStr">
-        <is>
-          <t>2026/08/06</t>
-        </is>
-      </c>
-      <c r="J53" s="9" t="inlineStr">
-        <is>
-          <t>2026/09/27</t>
-        </is>
-      </c>
-      <c r="K53" s="9" t="inlineStr">
-        <is>
-          <t>2027/01/11</t>
-        </is>
-      </c>
-      <c r="L53" s="9" t="inlineStr">
-        <is>
-          <t>2027/02/02</t>
-        </is>
-      </c>
-      <c r="M53" s="9" t="inlineStr">
-        <is>
-          <t>2027/03/08</t>
-        </is>
-      </c>
-      <c r="N53" s="9" t="inlineStr">
-        <is>
-          <t>2027/03/18</t>
-        </is>
-      </c>
-      <c r="O53" s="11" t="inlineStr">
-        <is>
-          <t>9/27 EVT SMT，9/28 Pre Assy，10/9 Assy</t>
-        </is>
-      </c>
-      <c r="P53" s="11" t="inlineStr">
+      <c r="P53" s="6" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -4674,7 +4660,7 @@
       </c>
       <c r="C54" s="9" t="inlineStr">
         <is>
-          <t>Crosshair 16 Max HX E4WGK</t>
+          <t>Crosshair 16 Max HX E4WFK</t>
         </is>
       </c>
       <c r="D54" s="14" t="inlineStr">
@@ -4689,7 +4675,7 @@
       </c>
       <c r="F54" s="9" t="inlineStr">
         <is>
-          <t>RTX 5070</t>
+          <t>RTX 5060</t>
         </is>
       </c>
       <c r="G54" s="9" t="inlineStr">
@@ -4754,230 +4740,230 @@
       </c>
       <c r="C55" s="9" t="inlineStr">
         <is>
+          <t>Crosshair 16 Max HX E4WGK</t>
+        </is>
+      </c>
+      <c r="D55" s="14" t="inlineStr">
+        <is>
+          <t>EVT</t>
+        </is>
+      </c>
+      <c r="E55" s="9" t="inlineStr">
+        <is>
+          <t>NVL-HX 55W</t>
+        </is>
+      </c>
+      <c r="F55" s="9" t="inlineStr">
+        <is>
+          <t>RTX 5070</t>
+        </is>
+      </c>
+      <c r="G55" s="9" t="inlineStr">
+        <is>
+          <t>鮑佩佩</t>
+        </is>
+      </c>
+      <c r="H55" s="9" t="inlineStr">
+        <is>
+          <t>2026/05/19</t>
+        </is>
+      </c>
+      <c r="I55" s="9" t="inlineStr">
+        <is>
+          <t>2026/08/06</t>
+        </is>
+      </c>
+      <c r="J55" s="9" t="inlineStr">
+        <is>
+          <t>2026/09/27</t>
+        </is>
+      </c>
+      <c r="K55" s="9" t="inlineStr">
+        <is>
+          <t>2027/01/11</t>
+        </is>
+      </c>
+      <c r="L55" s="9" t="inlineStr">
+        <is>
+          <t>2027/02/02</t>
+        </is>
+      </c>
+      <c r="M55" s="9" t="inlineStr">
+        <is>
+          <t>2027/03/08</t>
+        </is>
+      </c>
+      <c r="N55" s="9" t="inlineStr">
+        <is>
+          <t>2027/03/18</t>
+        </is>
+      </c>
+      <c r="O55" s="11" t="inlineStr">
+        <is>
+          <t>9/27 EVT SMT，9/28 Pre Assy，10/9 Assy</t>
+        </is>
+      </c>
+      <c r="P55" s="11" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" hidden="1" outlineLevel="1">
+      <c r="A56" s="7" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="8" t="inlineStr">
+        <is>
+          <t>2655</t>
+        </is>
+      </c>
+      <c r="C56" s="9" t="inlineStr">
+        <is>
           <t>Crosshair 16 Max HX E4WGXK</t>
         </is>
       </c>
-      <c r="D55" s="14" t="inlineStr">
+      <c r="D56" s="14" t="inlineStr">
         <is>
           <t>EVT</t>
         </is>
       </c>
-      <c r="E55" s="9" t="inlineStr">
+      <c r="E56" s="9" t="inlineStr">
         <is>
           <t>NVL-HX 55W</t>
         </is>
       </c>
-      <c r="F55" s="9" t="inlineStr">
+      <c r="F56" s="9" t="inlineStr">
         <is>
           <t>RTX 5070</t>
         </is>
       </c>
-      <c r="G55" s="9" t="inlineStr">
+      <c r="G56" s="9" t="inlineStr">
         <is>
           <t>鮑佩佩</t>
         </is>
       </c>
-      <c r="H55" s="9" t="inlineStr">
+      <c r="H56" s="9" t="inlineStr">
         <is>
           <t>2026/05/19</t>
         </is>
       </c>
-      <c r="I55" s="9" t="inlineStr">
+      <c r="I56" s="9" t="inlineStr">
         <is>
           <t>2026/08/06</t>
         </is>
       </c>
-      <c r="J55" s="9" t="inlineStr">
+      <c r="J56" s="9" t="inlineStr">
         <is>
           <t>2026/09/27</t>
         </is>
       </c>
-      <c r="K55" s="9" t="inlineStr">
+      <c r="K56" s="9" t="inlineStr">
         <is>
           <t>2027/01/11</t>
         </is>
       </c>
-      <c r="L55" s="9" t="inlineStr">
+      <c r="L56" s="9" t="inlineStr">
         <is>
           <t>2027/02/02</t>
         </is>
       </c>
-      <c r="M55" s="9" t="inlineStr">
+      <c r="M56" s="9" t="inlineStr">
         <is>
           <t>2027/03/08</t>
         </is>
       </c>
-      <c r="N55" s="9" t="inlineStr">
+      <c r="N56" s="9" t="inlineStr">
         <is>
           <t>2027/03/18</t>
         </is>
       </c>
-      <c r="O55" s="11" t="inlineStr">
+      <c r="O56" s="11" t="inlineStr">
         <is>
           <t>9/27 EVT SMT，9/28 Pre Assy，10/9 Assy</t>
         </is>
       </c>
-      <c r="P55" s="11" t="inlineStr">
+      <c r="P56" s="11" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="B56" s="3" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
         <is>
           <t>1862</t>
         </is>
       </c>
-      <c r="C56" s="4" t="inlineStr">
+      <c r="C57" s="4" t="inlineStr">
         <is>
           <t>Crosshair 18 Max HX B4WE</t>
         </is>
       </c>
-      <c r="D56" s="15" t="inlineStr">
+      <c r="D57" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
       </c>
-      <c r="E56" s="4" t="inlineStr">
+      <c r="E57" s="4" t="inlineStr">
         <is>
           <t>NVL-HX 55W</t>
         </is>
       </c>
-      <c r="F56" s="4" t="inlineStr">
+      <c r="F57" s="4" t="inlineStr">
         <is>
           <t>RTX 5050</t>
         </is>
       </c>
-      <c r="G56" s="4" t="inlineStr">
+      <c r="G57" s="4" t="inlineStr">
         <is>
           <t>劉芬</t>
         </is>
       </c>
-      <c r="H56" s="4" t="inlineStr">
+      <c r="H57" s="4" t="inlineStr">
         <is>
           <t>2026/08/21</t>
         </is>
       </c>
-      <c r="I56" s="4" t="inlineStr">
+      <c r="I57" s="4" t="inlineStr">
         <is>
           <t>2026/09/26</t>
         </is>
       </c>
-      <c r="J56" s="4" t="inlineStr">
+      <c r="J57" s="4" t="inlineStr">
         <is>
           <t>2026/12/07</t>
         </is>
       </c>
-      <c r="K56" s="4" t="inlineStr">
+      <c r="K57" s="4" t="inlineStr">
         <is>
           <t>2027/01/22</t>
         </is>
       </c>
-      <c r="L56" s="4" t="inlineStr">
+      <c r="L57" s="4" t="inlineStr">
         <is>
           <t>2027/03/03</t>
         </is>
       </c>
-      <c r="M56" s="4" t="inlineStr">
+      <c r="M57" s="4" t="inlineStr">
         <is>
           <t>2027/03/19</t>
         </is>
       </c>
-      <c r="N56" s="4" t="inlineStr">
+      <c r="N57" s="4" t="inlineStr">
         <is>
           <t>2027/03/30</t>
         </is>
       </c>
-      <c r="O56" s="6" t="inlineStr">
+      <c r="O57" s="6" t="inlineStr">
         <is>
           <t>1. PCB來料不足DVT分兩次打板，DVT-1 SMT 9/26 20pcs，DVT-2 SMT預排10/12 10pcs</t>
         </is>
       </c>
-      <c r="P56" s="6" t="inlineStr">
-        <is>
-          <t>1)Schedule：1862 schedule Pull in，TTM 3/E，update ATS 3/31==&gt;3/19，call help WHQL ready@3/30，gap 2W</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" hidden="1" outlineLevel="1">
-      <c r="A57" s="7" t="n">
-        <v>56</v>
-      </c>
-      <c r="B57" s="8" t="inlineStr">
-        <is>
-          <t>1862</t>
-        </is>
-      </c>
-      <c r="C57" s="9" t="inlineStr">
-        <is>
-          <t>Crosshair 18 Max HX B4WF</t>
-        </is>
-      </c>
-      <c r="D57" s="17" t="inlineStr">
-        <is>
-          <t>DVT</t>
-        </is>
-      </c>
-      <c r="E57" s="9" t="inlineStr">
-        <is>
-          <t>NVL-HX 55W</t>
-        </is>
-      </c>
-      <c r="F57" s="9" t="inlineStr">
-        <is>
-          <t>RTX 5060</t>
-        </is>
-      </c>
-      <c r="G57" s="9" t="inlineStr">
-        <is>
-          <t>劉芬</t>
-        </is>
-      </c>
-      <c r="H57" s="9" t="inlineStr">
-        <is>
-          <t>2026/08/21</t>
-        </is>
-      </c>
-      <c r="I57" s="9" t="inlineStr">
-        <is>
-          <t>2026/09/26</t>
-        </is>
-      </c>
-      <c r="J57" s="9" t="inlineStr">
-        <is>
-          <t>2026/12/07</t>
-        </is>
-      </c>
-      <c r="K57" s="9" t="inlineStr">
-        <is>
-          <t>2027/01/22</t>
-        </is>
-      </c>
-      <c r="L57" s="9" t="inlineStr">
-        <is>
-          <t>2027/03/03</t>
-        </is>
-      </c>
-      <c r="M57" s="9" t="inlineStr">
-        <is>
-          <t>2027/03/19</t>
-        </is>
-      </c>
-      <c r="N57" s="9" t="inlineStr">
-        <is>
-          <t>2027/03/30</t>
-        </is>
-      </c>
-      <c r="O57" s="11" t="inlineStr">
-        <is>
-          <t>1. PCB來料不足DVT分兩次打板，DVT-1 SMT 9/26 20pcs，DVT-2 SMT預排10/12 10pcs</t>
-        </is>
-      </c>
-      <c r="P57" s="11" t="inlineStr">
+      <c r="P57" s="6" t="inlineStr">
         <is>
           <t>1)Schedule：1862 schedule Pull in，TTM 3/E，update ATS 3/31==&gt;3/19，call help WHQL ready@3/30，gap 2W</t>
         </is>
@@ -4994,149 +4980,390 @@
       </c>
       <c r="C58" s="9" t="inlineStr">
         <is>
+          <t>Crosshair 18 Max HX B4WF</t>
+        </is>
+      </c>
+      <c r="D58" s="17" t="inlineStr">
+        <is>
+          <t>DVT</t>
+        </is>
+      </c>
+      <c r="E58" s="9" t="inlineStr">
+        <is>
+          <t>NVL-HX 55W</t>
+        </is>
+      </c>
+      <c r="F58" s="9" t="inlineStr">
+        <is>
+          <t>RTX 5060</t>
+        </is>
+      </c>
+      <c r="G58" s="9" t="inlineStr">
+        <is>
+          <t>劉芬</t>
+        </is>
+      </c>
+      <c r="H58" s="9" t="inlineStr">
+        <is>
+          <t>2026/08/21</t>
+        </is>
+      </c>
+      <c r="I58" s="9" t="inlineStr">
+        <is>
+          <t>2026/09/26</t>
+        </is>
+      </c>
+      <c r="J58" s="9" t="inlineStr">
+        <is>
+          <t>2026/12/07</t>
+        </is>
+      </c>
+      <c r="K58" s="9" t="inlineStr">
+        <is>
+          <t>2027/01/22</t>
+        </is>
+      </c>
+      <c r="L58" s="9" t="inlineStr">
+        <is>
+          <t>2027/03/03</t>
+        </is>
+      </c>
+      <c r="M58" s="9" t="inlineStr">
+        <is>
+          <t>2027/03/19</t>
+        </is>
+      </c>
+      <c r="N58" s="9" t="inlineStr">
+        <is>
+          <t>2027/03/30</t>
+        </is>
+      </c>
+      <c r="O58" s="11" t="inlineStr">
+        <is>
+          <t>1. PCB來料不足DVT分兩次打板，DVT-1 SMT 9/26 20pcs，DVT-2 SMT預排10/12 10pcs</t>
+        </is>
+      </c>
+      <c r="P58" s="11" t="inlineStr">
+        <is>
+          <t>1)Schedule：1862 schedule Pull in，TTM 3/E，update ATS 3/31==&gt;3/19，call help WHQL ready@3/30，gap 2W</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" hidden="1" outlineLevel="1">
+      <c r="A59" s="7" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="8" t="inlineStr">
+        <is>
+          <t>1862</t>
+        </is>
+      </c>
+      <c r="C59" s="9" t="inlineStr">
+        <is>
           <t>Crosshair 18 Max HX B4WG</t>
         </is>
       </c>
-      <c r="D58" s="17" t="inlineStr">
+      <c r="D59" s="17" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
       </c>
-      <c r="E58" s="9" t="inlineStr">
+      <c r="E59" s="9" t="inlineStr">
         <is>
           <t>NVL-HX 55W</t>
         </is>
       </c>
-      <c r="F58" s="9" t="inlineStr">
+      <c r="F59" s="9" t="inlineStr">
         <is>
           <t>RTX 5070</t>
         </is>
       </c>
-      <c r="G58" s="9" t="inlineStr">
+      <c r="G59" s="9" t="inlineStr">
         <is>
           <t>劉芬</t>
         </is>
       </c>
-      <c r="H58" s="9" t="inlineStr">
+      <c r="H59" s="9" t="inlineStr">
         <is>
           <t>2026/08/21</t>
         </is>
       </c>
-      <c r="I58" s="9" t="inlineStr">
+      <c r="I59" s="9" t="inlineStr">
         <is>
           <t>2026/09/26</t>
         </is>
       </c>
-      <c r="J58" s="9" t="inlineStr">
+      <c r="J59" s="9" t="inlineStr">
         <is>
           <t>2026/12/07</t>
         </is>
       </c>
-      <c r="K58" s="9" t="inlineStr">
+      <c r="K59" s="9" t="inlineStr">
         <is>
           <t>2027/01/22</t>
         </is>
       </c>
-      <c r="L58" s="9" t="inlineStr">
+      <c r="L59" s="9" t="inlineStr">
         <is>
           <t>2027/03/03</t>
         </is>
       </c>
-      <c r="M58" s="9" t="inlineStr">
+      <c r="M59" s="9" t="inlineStr">
         <is>
           <t>2027/03/19</t>
         </is>
       </c>
-      <c r="N58" s="9" t="inlineStr">
+      <c r="N59" s="9" t="inlineStr">
         <is>
           <t>2027/03/30</t>
         </is>
       </c>
-      <c r="O58" s="11" t="inlineStr">
+      <c r="O59" s="11" t="inlineStr">
         <is>
           <t>1. PCB來料不足DVT分兩次打板，DVT-1 SMT 9/26 20pcs，DVT-2 SMT預排10/12 10pcs</t>
         </is>
       </c>
-      <c r="P58" s="11" t="inlineStr">
+      <c r="P59" s="11" t="inlineStr">
         <is>
           <t>1)Schedule：1862 schedule Pull in，TTM 3/E，update ATS 3/31==&gt;3/19，call help WHQL ready@3/30，gap 2W</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="2" t="n">
-        <v>58</v>
-      </c>
-      <c r="B59" s="3" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
         <is>
           <t>2665</t>
         </is>
       </c>
-      <c r="C59" s="4" t="inlineStr">
+      <c r="C60" s="4" t="inlineStr">
         <is>
           <t>Cyborg N16 C1M</t>
         </is>
       </c>
-      <c r="D59" s="16" t="inlineStr">
+      <c r="D60" s="16" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
       </c>
-      <c r="E59" s="4" t="inlineStr">
+      <c r="E60" s="4" t="inlineStr">
         <is>
           <t>N1 45W</t>
         </is>
       </c>
-      <c r="F59" s="4" t="inlineStr">
+      <c r="F60" s="4" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="G59" s="4" t="inlineStr">
+      <c r="G60" s="4" t="inlineStr">
         <is>
           <t>梅燕</t>
         </is>
       </c>
-      <c r="H59" s="4" t="inlineStr">
+      <c r="H60" s="4" t="inlineStr">
         <is>
           <t>2026/09/30</t>
         </is>
       </c>
-      <c r="I59" s="4" t="inlineStr">
+      <c r="I60" s="4" t="inlineStr">
         <is>
           <t>2026/11/25</t>
         </is>
       </c>
-      <c r="J59" s="4" t="inlineStr">
+      <c r="J60" s="4" t="inlineStr">
         <is>
           <t>2026/12/16</t>
         </is>
       </c>
-      <c r="K59" s="4" t="inlineStr">
+      <c r="K60" s="4" t="inlineStr">
         <is>
           <t>2027/02/24</t>
         </is>
       </c>
-      <c r="L59" s="4" t="inlineStr">
+      <c r="L60" s="4" t="inlineStr">
         <is>
           <t>2027/03/01</t>
         </is>
       </c>
-      <c r="M59" s="4" t="inlineStr">
+      <c r="M60" s="4" t="inlineStr">
         <is>
           <t>2027/03/27</t>
         </is>
       </c>
-      <c r="N59" s="4" t="inlineStr">
+      <c r="N60" s="4" t="inlineStr">
         <is>
           <t>2027/04/09</t>
         </is>
       </c>
-      <c r="O59" s="6" t="inlineStr"/>
-      <c r="P59" s="6" t="inlineStr"/>
+      <c r="O60" s="6" t="inlineStr"/>
+      <c r="P60" s="6" t="inlineStr">
+        <is>
+          <t>1).待NV 更新65W 設計 , 評估是否重新 kick off
+2).schedule 待調整</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>2663</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>Stealth 16S C4M</t>
+        </is>
+      </c>
+      <c r="D61" s="16" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="inlineStr">
+        <is>
+          <t>NVL-H 45W</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>Intel® Arc™ Graphics</t>
+        </is>
+      </c>
+      <c r="G61" s="4" t="inlineStr">
+        <is>
+          <t>鮑佩佩</t>
+        </is>
+      </c>
+      <c r="H61" s="4" t="inlineStr">
+        <is>
+          <t>2026/10/13</t>
+        </is>
+      </c>
+      <c r="I61" s="4" t="inlineStr">
+        <is>
+          <t>2026/12/02</t>
+        </is>
+      </c>
+      <c r="J61" s="4" t="inlineStr">
+        <is>
+          <t>2027/01/18</t>
+        </is>
+      </c>
+      <c r="K61" s="4" t="inlineStr">
+        <is>
+          <t>2027/03/09</t>
+        </is>
+      </c>
+      <c r="L61" s="4" t="inlineStr">
+        <is>
+          <t>2027/04/02</t>
+        </is>
+      </c>
+      <c r="M61" s="4" t="inlineStr">
+        <is>
+          <t>2027/04/30</t>
+        </is>
+      </c>
+      <c r="N61" s="4" t="inlineStr">
+        <is>
+          <t>2027/05/15</t>
+        </is>
+      </c>
+      <c r="O61" s="6" t="inlineStr">
+        <is>
+          <t>10/20-11/17 0A layout</t>
+        </is>
+      </c>
+      <c r="P61" s="6" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>2664</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>Prestige N16S AI+ D1XMT</t>
+        </is>
+      </c>
+      <c r="D62" s="16" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="inlineStr">
+        <is>
+          <t>N1x 80W</t>
+        </is>
+      </c>
+      <c r="F62" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G62" s="4" t="inlineStr">
+        <is>
+          <t>李文欽</t>
+        </is>
+      </c>
+      <c r="H62" s="4" t="inlineStr">
+        <is>
+          <t>2026/10/14</t>
+        </is>
+      </c>
+      <c r="I62" s="4" t="inlineStr">
+        <is>
+          <t>2026/12/22</t>
+        </is>
+      </c>
+      <c r="J62" s="4" t="inlineStr">
+        <is>
+          <t>2027/01/19</t>
+        </is>
+      </c>
+      <c r="K62" s="4" t="inlineStr">
+        <is>
+          <t>2027/03/26</t>
+        </is>
+      </c>
+      <c r="L62" s="4" t="inlineStr">
+        <is>
+          <t>2027/04/08</t>
+        </is>
+      </c>
+      <c r="M62" s="4" t="inlineStr">
+        <is>
+          <t>2027/05/06</t>
+        </is>
+      </c>
+      <c r="N62" s="4" t="inlineStr">
+        <is>
+          <t>2027/05/19</t>
+        </is>
+      </c>
+      <c r="O62" s="6" t="inlineStr"/>
+      <c r="P62" s="6" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P59"/>
+  <autoFilter ref="A1:P62"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update NPI Dashboard 2026-10-22 17:27
</commit_message>
<xml_diff>
--- a/npi_dashboard.xlsx
+++ b/npi_dashboard.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Raider A16 HX B9WI</t>
+          <t>Raider A16 HX B9WH</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
@@ -708,7 +708,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>RTX 5080</t>
+          <t>RTX 5070Ti</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -751,7 +751,9 @@
       </c>
       <c r="P3" s="6" t="inlineStr">
         <is>
-          <t>無.</t>
+          <t>Schedule:MVT Gating Issue需RD於10/28前導入solution
+1). 單/雙燒GPU TDP足瓦175W不穩定，10s即開始降頻
+2). 同時外接2個TBT monitor會出現單屏不顯/hang up等多種異常</t>
         </is>
       </c>
     </row>
@@ -766,7 +768,7 @@
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>Raider A16 HX B9WJ</t>
+          <t>Raider A16 HX B9WI</t>
         </is>
       </c>
       <c r="D4" s="10" t="inlineStr">
@@ -781,7 +783,7 @@
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>RTX 5090</t>
+          <t>RTX 5080</t>
         </is>
       </c>
       <c r="G4" s="9" t="inlineStr">
@@ -824,7 +826,9 @@
       </c>
       <c r="P4" s="11" t="inlineStr">
         <is>
-          <t>無.</t>
+          <t>Schedule:MVT Gating Issue需RD於10/28前導入solution
+1). 單/雙燒GPU TDP足瓦175W不穩定，10s即開始降頻
+2). 同時外接2個TBT monitor會出現單屏不顯/hang up等多種異常</t>
         </is>
       </c>
     </row>
@@ -839,7 +843,7 @@
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>Raider A16 HX B9WH</t>
+          <t>Raider A16 HX B9WJ</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
@@ -854,7 +858,7 @@
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
-          <t>RTX 5070Ti</t>
+          <t>RTX 5090</t>
         </is>
       </c>
       <c r="G5" s="9" t="inlineStr">
@@ -897,7 +901,9 @@
       </c>
       <c r="P5" s="11" t="inlineStr">
         <is>
-          <t>無</t>
+          <t>Schedule:MVT Gating Issue需RD於10/28前導入solution
+1). 單/雙燒GPU TDP足瓦175W不穩定，10s即開始降頻
+2). 同時外接2個TBT monitor會出現單屏不顯/hang up等多種異常</t>
         </is>
       </c>
     </row>
@@ -2769,8 +2775,7 @@
       </c>
       <c r="P30" s="6" t="inlineStr">
         <is>
-          <t>1)備料：a. 2.8K panel: SDC update因PCB物料短缺會delay至11/M ETD, 影響2nd MP時間約1 week , 仍在請廠商pull in中
-2）Schedule: NV FD software時間可能會delay到week 12/14, 預抓1 week準備Software, 2 weeks DQA測試後, 1/11 ATS start</t>
+          <t>1) Schedule update: NV FD software時間可能會delay到week 12/14, 預抓1 week準備Software, 2 weeks DQA測試後, 1/11 ATS start</t>
         </is>
       </c>
     </row>
@@ -3428,12 +3433,12 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>13Q5</t>
+          <t>2633</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Prestige 13 AI+ A4M</t>
+          <t>Stealth 16 AI+ B4WI</t>
         </is>
       </c>
       <c r="D40" s="15" t="inlineStr">
@@ -3443,147 +3448,142 @@
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>NVL-H 28W</t>
+          <t>NVL-H 45W</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>Intel® Arc™ Graphics</t>
+          <t>RTX 5080</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>顏春梅</t>
+          <t>朱欣怡</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>2026/06/29</t>
+          <t>2026/05/22</t>
         </is>
       </c>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>2026/08/18</t>
+          <t>2026/07/23</t>
         </is>
       </c>
       <c r="J40" s="4" t="inlineStr">
         <is>
-          <t>2026/10/10</t>
+          <t>2026/09/16</t>
         </is>
       </c>
       <c r="K40" s="4" t="inlineStr">
         <is>
-          <t>2026/12/03</t>
+          <t>2026/12/02</t>
         </is>
       </c>
       <c r="L40" s="4" t="inlineStr">
         <is>
-          <t>2026/12/25</t>
+          <t>2027/01/15</t>
         </is>
       </c>
       <c r="M40" s="4" t="inlineStr">
         <is>
-          <t>2027/01/26</t>
+          <t>2027/02/16</t>
         </is>
       </c>
       <c r="N40" s="4" t="inlineStr">
         <is>
-          <t>2027/02/05</t>
+          <t>2027/02/26</t>
         </is>
       </c>
       <c r="O40" s="6" t="inlineStr">
         <is>
-          <t>EVT 機台10/20調撥回台 預計23號 RD 開始測試</t>
+          <t>DQA 測試中</t>
         </is>
       </c>
       <c r="P40" s="6" t="inlineStr">
         <is>
-          <t>1.NPI schedule: ATS for 16C/14C/8C(1/26~2/5 RD&amp;工廠春節需配合加班，海關放假影響出貨） 2.备料: MVT DQA 測試一周需PCB risk buy 3.软体:TBT sign FW Gap 4W(PV SW release@ WW03-05’27 FV 無測試時間) 4.認證:N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="n">
+          <t>1）TBT FV test:1/27~2/23, 與 ATS 2/16 gating  1 Week</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" hidden="1" outlineLevel="1">
+      <c r="A41" s="7" t="n">
         <v>40</v>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B41" s="8" t="inlineStr">
         <is>
           <t>2633</t>
         </is>
       </c>
-      <c r="C41" s="4" t="inlineStr">
-        <is>
-          <t>Stealth 16 AI+ B4WI</t>
-        </is>
-      </c>
-      <c r="D41" s="15" t="inlineStr">
+      <c r="C41" s="9" t="inlineStr">
+        <is>
+          <t>Stealth 16 AI+ B4WH</t>
+        </is>
+      </c>
+      <c r="D41" s="16" t="inlineStr">
         <is>
           <t>EVT</t>
         </is>
       </c>
-      <c r="E41" s="4" t="inlineStr">
+      <c r="E41" s="9" t="inlineStr">
         <is>
           <t>NVL-H 45W</t>
         </is>
       </c>
-      <c r="F41" s="4" t="inlineStr">
-        <is>
-          <t>RTX 5080</t>
-        </is>
-      </c>
-      <c r="G41" s="4" t="inlineStr">
+      <c r="F41" s="9" t="inlineStr">
+        <is>
+          <t>RTX 5070Ti</t>
+        </is>
+      </c>
+      <c r="G41" s="9" t="inlineStr">
         <is>
           <t>朱欣怡</t>
         </is>
       </c>
-      <c r="H41" s="4" t="inlineStr">
+      <c r="H41" s="9" t="inlineStr">
         <is>
           <t>2026/05/22</t>
         </is>
       </c>
-      <c r="I41" s="4" t="inlineStr">
+      <c r="I41" s="9" t="inlineStr">
         <is>
           <t>2026/07/23</t>
         </is>
       </c>
-      <c r="J41" s="4" t="inlineStr">
+      <c r="J41" s="9" t="inlineStr">
         <is>
           <t>2026/09/16</t>
         </is>
       </c>
-      <c r="K41" s="4" t="inlineStr">
+      <c r="K41" s="9" t="inlineStr">
         <is>
           <t>2026/12/02</t>
         </is>
       </c>
-      <c r="L41" s="4" t="inlineStr">
+      <c r="L41" s="9" t="inlineStr">
         <is>
           <t>2027/01/15</t>
         </is>
       </c>
-      <c r="M41" s="4" t="inlineStr">
+      <c r="M41" s="9" t="inlineStr">
         <is>
           <t>2027/02/16</t>
         </is>
       </c>
-      <c r="N41" s="4" t="inlineStr">
+      <c r="N41" s="9" t="inlineStr">
         <is>
           <t>2027/02/26</t>
         </is>
       </c>
-      <c r="O41" s="6" t="inlineStr">
+      <c r="O41" s="11" t="inlineStr">
         <is>
           <t>DQA 測試中</t>
         </is>
       </c>
-      <c r="P41" s="6" t="inlineStr">
-        <is>
-          <t>若要pull in ATS @1/26：
-1）NV VBIOS 完成@2/2, 與 ATS 1/26 gating 1 Week；
-2）TBT FV test:1/27~2/23, 與 ATS 1/26 gating  4 Weeks；
-3）Thermal EVT 測試完需備料for ATS；
-4）MVT DQA 測試一周需PCB risk buy （WW
-52）</t>
+      <c r="P41" s="11" t="inlineStr">
+        <is>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -3598,7 +3598,7 @@
       </c>
       <c r="C42" s="9" t="inlineStr">
         <is>
-          <t>Stealth 16 AI+ B4WH</t>
+          <t>Stealth 16 AI+ B4WJ</t>
         </is>
       </c>
       <c r="D42" s="16" t="inlineStr">
@@ -3613,7 +3613,7 @@
       </c>
       <c r="F42" s="9" t="inlineStr">
         <is>
-          <t>RTX 5070Ti</t>
+          <t>RTX 5090</t>
         </is>
       </c>
       <c r="G42" s="9" t="inlineStr">
@@ -3667,168 +3667,163 @@
         </is>
       </c>
     </row>
-    <row r="43" hidden="1" outlineLevel="1">
-      <c r="A43" s="7" t="n">
+    <row r="43">
+      <c r="A43" s="2" t="n">
         <v>42</v>
       </c>
-      <c r="B43" s="8" t="inlineStr">
-        <is>
-          <t>2633</t>
-        </is>
-      </c>
-      <c r="C43" s="9" t="inlineStr">
-        <is>
-          <t>Stealth 16 AI+ B4WJ</t>
-        </is>
-      </c>
-      <c r="D43" s="16" t="inlineStr">
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>2634</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Stealth 16 AI+ B4WE</t>
+        </is>
+      </c>
+      <c r="D43" s="15" t="inlineStr">
         <is>
           <t>EVT</t>
         </is>
       </c>
-      <c r="E43" s="9" t="inlineStr">
+      <c r="E43" s="4" t="inlineStr">
         <is>
           <t>NVL-H 45W</t>
         </is>
       </c>
-      <c r="F43" s="9" t="inlineStr">
-        <is>
-          <t>RTX 5090</t>
-        </is>
-      </c>
-      <c r="G43" s="9" t="inlineStr">
-        <is>
-          <t>朱欣怡</t>
-        </is>
-      </c>
-      <c r="H43" s="9" t="inlineStr">
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>RTX 5050</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>賴雪鳳</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="inlineStr">
         <is>
           <t>2026/05/22</t>
         </is>
       </c>
-      <c r="I43" s="9" t="inlineStr">
-        <is>
-          <t>2026/07/23</t>
-        </is>
-      </c>
-      <c r="J43" s="9" t="inlineStr">
-        <is>
-          <t>2026/09/16</t>
-        </is>
-      </c>
-      <c r="K43" s="9" t="inlineStr">
+      <c r="I43" s="4" t="inlineStr">
+        <is>
+          <t>2026/07/31</t>
+        </is>
+      </c>
+      <c r="J43" s="4" t="inlineStr">
+        <is>
+          <t>2026/09/17</t>
+        </is>
+      </c>
+      <c r="K43" s="4" t="inlineStr">
         <is>
           <t>2026/12/02</t>
         </is>
       </c>
-      <c r="L43" s="9" t="inlineStr">
-        <is>
-          <t>2027/01/15</t>
-        </is>
-      </c>
-      <c r="M43" s="9" t="inlineStr">
+      <c r="L43" s="4" t="inlineStr">
+        <is>
+          <t>2027/01/13</t>
+        </is>
+      </c>
+      <c r="M43" s="4" t="inlineStr">
         <is>
           <t>2027/02/16</t>
         </is>
       </c>
-      <c r="N43" s="9" t="inlineStr">
+      <c r="N43" s="4" t="inlineStr">
         <is>
           <t>2027/02/26</t>
         </is>
       </c>
-      <c r="O43" s="11" t="inlineStr">
-        <is>
-          <t>DQA 測試中</t>
-        </is>
-      </c>
-      <c r="P43" s="11" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="n">
+      <c r="O43" s="6" t="inlineStr">
+        <is>
+          <t>EVT驗證中</t>
+        </is>
+      </c>
+      <c r="P43" s="6" t="inlineStr">
+        <is>
+          <t>1）TBT FV test:1/27~2/23, 與 ATS 2/16 gating 1 Week</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" hidden="1" outlineLevel="1">
+      <c r="A44" s="7" t="n">
         <v>43</v>
       </c>
-      <c r="B44" s="3" t="inlineStr">
+      <c r="B44" s="8" t="inlineStr">
         <is>
           <t>2634</t>
         </is>
       </c>
-      <c r="C44" s="4" t="inlineStr">
-        <is>
-          <t>Stealth 16 AI+ B4WE</t>
-        </is>
-      </c>
-      <c r="D44" s="15" t="inlineStr">
+      <c r="C44" s="9" t="inlineStr">
+        <is>
+          <t>Stealth 16 AI+ B4WF</t>
+        </is>
+      </c>
+      <c r="D44" s="16" t="inlineStr">
         <is>
           <t>EVT</t>
         </is>
       </c>
-      <c r="E44" s="4" t="inlineStr">
+      <c r="E44" s="9" t="inlineStr">
         <is>
           <t>NVL-H 45W</t>
         </is>
       </c>
-      <c r="F44" s="4" t="inlineStr">
-        <is>
-          <t>RTX 5050</t>
-        </is>
-      </c>
-      <c r="G44" s="4" t="inlineStr">
+      <c r="F44" s="9" t="inlineStr">
+        <is>
+          <t>RTX 5060</t>
+        </is>
+      </c>
+      <c r="G44" s="9" t="inlineStr">
         <is>
           <t>賴雪鳳</t>
         </is>
       </c>
-      <c r="H44" s="4" t="inlineStr">
+      <c r="H44" s="9" t="inlineStr">
         <is>
           <t>2026/05/22</t>
         </is>
       </c>
-      <c r="I44" s="4" t="inlineStr">
+      <c r="I44" s="9" t="inlineStr">
         <is>
           <t>2026/07/31</t>
         </is>
       </c>
-      <c r="J44" s="4" t="inlineStr">
+      <c r="J44" s="9" t="inlineStr">
         <is>
           <t>2026/09/17</t>
         </is>
       </c>
-      <c r="K44" s="4" t="inlineStr">
+      <c r="K44" s="9" t="inlineStr">
         <is>
           <t>2026/12/02</t>
         </is>
       </c>
-      <c r="L44" s="4" t="inlineStr">
+      <c r="L44" s="9" t="inlineStr">
         <is>
           <t>2027/01/13</t>
         </is>
       </c>
-      <c r="M44" s="4" t="inlineStr">
+      <c r="M44" s="9" t="inlineStr">
         <is>
           <t>2027/02/16</t>
         </is>
       </c>
-      <c r="N44" s="4" t="inlineStr">
+      <c r="N44" s="9" t="inlineStr">
         <is>
           <t>2027/02/26</t>
         </is>
       </c>
-      <c r="O44" s="6" t="inlineStr">
+      <c r="O44" s="11" t="inlineStr">
         <is>
           <t>EVT驗證中</t>
         </is>
       </c>
-      <c r="P44" s="6" t="inlineStr">
-        <is>
-          <t>若要pull in ATS @1/26：
-1）NV VBIOS 完成@2/2, 與 ATS 1/26 gating 1 Week；
-2）TBT FV test:1/27~2/23, 與 ATS 1/26 gating 4 Weeks；
-3）Thermal EVT 測試完需備料for ATS；
-4）MVT DQA 測試一周需PCB risk buy （WW
-52）</t>
+      <c r="P44" s="11" t="inlineStr">
+        <is>
+          <t>1）TBT FV test:1/27~2/23, 與 ATS 2/16 gating 1 Week</t>
         </is>
       </c>
     </row>
@@ -3843,7 +3838,7 @@
       </c>
       <c r="C45" s="9" t="inlineStr">
         <is>
-          <t>Stealth 16 AI+ B4WF</t>
+          <t>Stealth 16 AI+ B4WG/GD7 8GB</t>
         </is>
       </c>
       <c r="D45" s="16" t="inlineStr">
@@ -3858,7 +3853,7 @@
       </c>
       <c r="F45" s="9" t="inlineStr">
         <is>
-          <t>RTX 5060</t>
+          <t>RTX 5070</t>
         </is>
       </c>
       <c r="G45" s="9" t="inlineStr">
@@ -3903,17 +3898,12 @@
       </c>
       <c r="O45" s="11" t="inlineStr">
         <is>
-          <t>EVT驗證中</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="P45" s="11" t="inlineStr">
         <is>
-          <t>若要pull in ATS @1/26：
-1）NV VBIOS 完成@2/2, 與 ATS 1/26 gating 1 Week；
-2）TBT FV test:1/27~2/23, 與 ATS 1/26 gating 4 Weeks；
-3）Thermal EVT 測試完需備料for ATS；
-4）MVT DQA 測試一周需PCB risk buy （WW
-52）</t>
+          <t>1）TBT FV test:1/27~2/23, 與 ATS 2/16 gating 1 Week</t>
         </is>
       </c>
     </row>
@@ -3928,7 +3918,7 @@
       </c>
       <c r="C46" s="9" t="inlineStr">
         <is>
-          <t>Stealth 16 AI+ B4WG/GD7 8GB</t>
+          <t>Stealth 16 AI+ B4WGX/GD7 12GB</t>
         </is>
       </c>
       <c r="D46" s="16" t="inlineStr">
@@ -3988,414 +3978,404 @@
       </c>
       <c r="O46" s="11" t="inlineStr">
         <is>
+          <t>EVT驗證中</t>
+        </is>
+      </c>
+      <c r="P46" s="11" t="inlineStr">
+        <is>
+          <t>1）TBT FV test:1/27~2/23, 與 ATS 2/16 gating 1 Week</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>14T4</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>Prestige 14 AI+ D4M</t>
+        </is>
+      </c>
+      <c r="D47" s="15" t="inlineStr">
+        <is>
+          <t>EVT</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>NVL-H 30W</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>Intel® Arc™ Graphics</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>朱芳芳</t>
+        </is>
+      </c>
+      <c r="H47" s="4" t="inlineStr">
+        <is>
+          <t>2026/05/14</t>
+        </is>
+      </c>
+      <c r="I47" s="4" t="inlineStr">
+        <is>
+          <t>2026/07/27</t>
+        </is>
+      </c>
+      <c r="J47" s="4" t="inlineStr">
+        <is>
+          <t>2026/10/17</t>
+        </is>
+      </c>
+      <c r="K47" s="4" t="inlineStr">
+        <is>
+          <t>2026/12/02</t>
+        </is>
+      </c>
+      <c r="L47" s="4" t="inlineStr">
+        <is>
+          <t>2026/12/30</t>
+        </is>
+      </c>
+      <c r="M47" s="4" t="inlineStr">
+        <is>
+          <t>2027/02/16</t>
+        </is>
+      </c>
+      <c r="N47" s="4" t="inlineStr">
+        <is>
+          <t>2027/02/26</t>
+        </is>
+      </c>
+      <c r="O47" s="6" t="inlineStr">
+        <is>
+          <t>EVT組裝中，DQA test10/26～11/16</t>
+        </is>
+      </c>
+      <c r="P47" s="6" t="inlineStr">
+        <is>
+          <t>PCB 1.0  for MVT 需采購pull in 11/30 ready (3W 進料,LT：4W）</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" hidden="1" outlineLevel="1">
+      <c r="A48" s="7" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="8" t="inlineStr">
+        <is>
+          <t>14T4</t>
+        </is>
+      </c>
+      <c r="C48" s="9" t="inlineStr">
+        <is>
+          <t>Prestige 14 Flip AI+ D4MT</t>
+        </is>
+      </c>
+      <c r="D48" s="16" t="inlineStr">
+        <is>
+          <t>EVT</t>
+        </is>
+      </c>
+      <c r="E48" s="9" t="inlineStr">
+        <is>
+          <t>NVL-H 30W</t>
+        </is>
+      </c>
+      <c r="F48" s="9" t="inlineStr">
+        <is>
+          <t>Intel® Arc™ Graphics</t>
+        </is>
+      </c>
+      <c r="G48" s="9" t="inlineStr">
+        <is>
+          <t>朱芳芳</t>
+        </is>
+      </c>
+      <c r="H48" s="9" t="inlineStr">
+        <is>
+          <t>2026/05/14</t>
+        </is>
+      </c>
+      <c r="I48" s="9" t="inlineStr">
+        <is>
+          <t>2026/07/27</t>
+        </is>
+      </c>
+      <c r="J48" s="9" t="inlineStr">
+        <is>
+          <t>2026/10/17</t>
+        </is>
+      </c>
+      <c r="K48" s="9" t="inlineStr">
+        <is>
+          <t>2026/12/02</t>
+        </is>
+      </c>
+      <c r="L48" s="9" t="inlineStr">
+        <is>
+          <t>2026/12/30</t>
+        </is>
+      </c>
+      <c r="M48" s="9" t="inlineStr">
+        <is>
+          <t>2027/02/16</t>
+        </is>
+      </c>
+      <c r="N48" s="9" t="inlineStr">
+        <is>
+          <t>2027/02/26</t>
+        </is>
+      </c>
+      <c r="O48" s="11" t="inlineStr">
+        <is>
+          <t>EVT組裝中，DQA test10/26～11/16</t>
+        </is>
+      </c>
+      <c r="P48" s="11" t="inlineStr">
+        <is>
+          <t>PCB 1.0  for MVT 需采購pull in 11/30 ready (3W 進料,LT：4W）</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>2624</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>Prestige 16 AI+ C4M</t>
+        </is>
+      </c>
+      <c r="D49" s="15" t="inlineStr">
+        <is>
+          <t>EVT</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>NVL-H 30W</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>Intel® Arc™ Graphics</t>
+        </is>
+      </c>
+      <c r="G49" s="4" t="inlineStr">
+        <is>
+          <t>朱芳芳</t>
+        </is>
+      </c>
+      <c r="H49" s="4" t="inlineStr">
+        <is>
+          <t>2026/05/14</t>
+        </is>
+      </c>
+      <c r="I49" s="4" t="inlineStr"/>
+      <c r="J49" s="4" t="inlineStr">
+        <is>
+          <t>2026/10/17</t>
+        </is>
+      </c>
+      <c r="K49" s="4" t="inlineStr">
+        <is>
+          <t>2026/12/02</t>
+        </is>
+      </c>
+      <c r="L49" s="4" t="inlineStr">
+        <is>
+          <t>2026/12/30</t>
+        </is>
+      </c>
+      <c r="M49" s="4" t="inlineStr">
+        <is>
+          <t>2027/02/16</t>
+        </is>
+      </c>
+      <c r="N49" s="4" t="inlineStr">
+        <is>
+          <t>2027/02/26</t>
+        </is>
+      </c>
+      <c r="O49" s="6" t="inlineStr">
+        <is>
+          <t>EVT組裝中，DQA test10/26～11/16</t>
+        </is>
+      </c>
+      <c r="P49" s="6" t="inlineStr">
+        <is>
+          <t>PCB 1.0  for MVT 需采購pull in 11/30 ready (3W 進料,LT：4W）</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" hidden="1" outlineLevel="1">
+      <c r="A50" s="7" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="8" t="inlineStr">
+        <is>
+          <t>2624</t>
+        </is>
+      </c>
+      <c r="C50" s="9" t="inlineStr">
+        <is>
+          <t>Prestige 16 Flip AI+ C4MT</t>
+        </is>
+      </c>
+      <c r="D50" s="16" t="inlineStr">
+        <is>
+          <t>EVT</t>
+        </is>
+      </c>
+      <c r="E50" s="9" t="inlineStr">
+        <is>
+          <t>NVL-H 30W</t>
+        </is>
+      </c>
+      <c r="F50" s="9" t="inlineStr">
+        <is>
+          <t>Intel® Arc™ Graphics</t>
+        </is>
+      </c>
+      <c r="G50" s="9" t="inlineStr">
+        <is>
+          <t>朱芳芳</t>
+        </is>
+      </c>
+      <c r="H50" s="9" t="inlineStr">
+        <is>
+          <t>2026/05/14</t>
+        </is>
+      </c>
+      <c r="I50" s="9" t="inlineStr"/>
+      <c r="J50" s="9" t="inlineStr">
+        <is>
+          <t>2026/10/17</t>
+        </is>
+      </c>
+      <c r="K50" s="9" t="inlineStr">
+        <is>
+          <t>2026/12/02</t>
+        </is>
+      </c>
+      <c r="L50" s="9" t="inlineStr">
+        <is>
+          <t>2026/12/30</t>
+        </is>
+      </c>
+      <c r="M50" s="9" t="inlineStr">
+        <is>
+          <t>2027/02/16</t>
+        </is>
+      </c>
+      <c r="N50" s="9" t="inlineStr">
+        <is>
+          <t>2027/02/26</t>
+        </is>
+      </c>
+      <c r="O50" s="11" t="inlineStr">
+        <is>
+          <t>EVT組裝中，DQA test10/26～11/16</t>
+        </is>
+      </c>
+      <c r="P50" s="11" t="inlineStr">
+        <is>
+          <t>PCB 1.0  for MVT 需采購pull in 11/30 ready (3W 進料,LT：4W）</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>14W2</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>Prestige 14S E4M</t>
+        </is>
+      </c>
+      <c r="D51" s="14" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>NVL-H 30W</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>Intel® Arc™ Graphics</t>
+        </is>
+      </c>
+      <c r="G51" s="4" t="inlineStr">
+        <is>
+          <t>吳美芳</t>
+        </is>
+      </c>
+      <c r="H51" s="4" t="inlineStr">
+        <is>
+          <t>2026/09/11</t>
+        </is>
+      </c>
+      <c r="I51" s="4" t="inlineStr">
+        <is>
+          <t>2026/10/31</t>
+        </is>
+      </c>
+      <c r="J51" s="4" t="inlineStr">
+        <is>
+          <t>2026/12/13</t>
+        </is>
+      </c>
+      <c r="K51" s="4" t="inlineStr">
+        <is>
+          <t>2027/01/14</t>
+        </is>
+      </c>
+      <c r="L51" s="4" t="inlineStr">
+        <is>
+          <t>2027/01/21</t>
+        </is>
+      </c>
+      <c r="M51" s="4" t="inlineStr">
+        <is>
+          <t>2027/02/18</t>
+        </is>
+      </c>
+      <c r="N51" s="4" t="inlineStr">
+        <is>
+          <t>2027/02/28</t>
+        </is>
+      </c>
+      <c r="O51" s="6" t="inlineStr">
+        <is>
+          <t>10/22出图，DVT从11/4提前至10/31，后续schedule暂keep</t>
+        </is>
+      </c>
+      <c r="P51" s="6" t="inlineStr">
+        <is>
           <t>NA</t>
-        </is>
-      </c>
-      <c r="P46" s="11" t="inlineStr">
-        <is>
-          <t>若要pull in ATS @1/26：
-1）NV VBIOS 完成@2/2, 與 ATS 1/26 gating 1 Week；
-2）TBT FV test:1/27~2/23, 與 ATS 1/26 gating 4 Weeks；
-3）Thermal EVT 測試完需備料for ATS；
-4）MVT DQA 測試一周需PCB risk buy （WW
-52）</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" hidden="1" outlineLevel="1">
-      <c r="A47" s="7" t="n">
-        <v>46</v>
-      </c>
-      <c r="B47" s="8" t="inlineStr">
-        <is>
-          <t>2634</t>
-        </is>
-      </c>
-      <c r="C47" s="9" t="inlineStr">
-        <is>
-          <t>Stealth 16 AI+ B4WGX/GD7 12GB</t>
-        </is>
-      </c>
-      <c r="D47" s="16" t="inlineStr">
-        <is>
-          <t>EVT</t>
-        </is>
-      </c>
-      <c r="E47" s="9" t="inlineStr">
-        <is>
-          <t>NVL-H 45W</t>
-        </is>
-      </c>
-      <c r="F47" s="9" t="inlineStr">
-        <is>
-          <t>RTX 5070</t>
-        </is>
-      </c>
-      <c r="G47" s="9" t="inlineStr">
-        <is>
-          <t>賴雪鳳</t>
-        </is>
-      </c>
-      <c r="H47" s="9" t="inlineStr">
-        <is>
-          <t>2026/05/22</t>
-        </is>
-      </c>
-      <c r="I47" s="9" t="inlineStr">
-        <is>
-          <t>2026/07/31</t>
-        </is>
-      </c>
-      <c r="J47" s="9" t="inlineStr">
-        <is>
-          <t>2026/09/17</t>
-        </is>
-      </c>
-      <c r="K47" s="9" t="inlineStr">
-        <is>
-          <t>2026/12/02</t>
-        </is>
-      </c>
-      <c r="L47" s="9" t="inlineStr">
-        <is>
-          <t>2027/01/13</t>
-        </is>
-      </c>
-      <c r="M47" s="9" t="inlineStr">
-        <is>
-          <t>2027/02/16</t>
-        </is>
-      </c>
-      <c r="N47" s="9" t="inlineStr">
-        <is>
-          <t>2027/02/26</t>
-        </is>
-      </c>
-      <c r="O47" s="11" t="inlineStr">
-        <is>
-          <t>EVT驗證中</t>
-        </is>
-      </c>
-      <c r="P47" s="11" t="inlineStr">
-        <is>
-          <t>若要pull in ATS @1/26：
-1）NV VBIOS 完成@2/2, 與 ATS 1/26 gating 1 Week；
-2）TBT FV test:1/27~2/23, 與 ATS 1/26 gating 4 Weeks；
-3）Thermal EVT 測試完需備料for ATS；
-4）MVT DQA 測試一周需PCB risk buy （WW
-52）</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="n">
-        <v>47</v>
-      </c>
-      <c r="B48" s="3" t="inlineStr">
-        <is>
-          <t>14T4</t>
-        </is>
-      </c>
-      <c r="C48" s="4" t="inlineStr">
-        <is>
-          <t>Prestige 14 AI+ D4M</t>
-        </is>
-      </c>
-      <c r="D48" s="15" t="inlineStr">
-        <is>
-          <t>EVT</t>
-        </is>
-      </c>
-      <c r="E48" s="4" t="inlineStr">
-        <is>
-          <t>NVL-H 30W</t>
-        </is>
-      </c>
-      <c r="F48" s="4" t="inlineStr">
-        <is>
-          <t>Intel® Arc™ Graphics</t>
-        </is>
-      </c>
-      <c r="G48" s="4" t="inlineStr">
-        <is>
-          <t>朱芳芳</t>
-        </is>
-      </c>
-      <c r="H48" s="4" t="inlineStr">
-        <is>
-          <t>2026/05/14</t>
-        </is>
-      </c>
-      <c r="I48" s="4" t="inlineStr">
-        <is>
-          <t>2026/07/27</t>
-        </is>
-      </c>
-      <c r="J48" s="4" t="inlineStr">
-        <is>
-          <t>2026/10/17</t>
-        </is>
-      </c>
-      <c r="K48" s="4" t="inlineStr">
-        <is>
-          <t>2026/12/02</t>
-        </is>
-      </c>
-      <c r="L48" s="4" t="inlineStr">
-        <is>
-          <t>2026/12/30</t>
-        </is>
-      </c>
-      <c r="M48" s="4" t="inlineStr">
-        <is>
-          <t>2027/02/16</t>
-        </is>
-      </c>
-      <c r="N48" s="4" t="inlineStr">
-        <is>
-          <t>2027/02/26</t>
-        </is>
-      </c>
-      <c r="O48" s="6" t="inlineStr">
-        <is>
-          <t>EVT組裝中，DQA test12/26～11/16</t>
-        </is>
-      </c>
-      <c r="P48" s="6" t="inlineStr">
-        <is>
-          <t>PCB 1.0  for MVT 需采購pull in 11/30 ready (3W 進料,LT：4W）</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" hidden="1" outlineLevel="1">
-      <c r="A49" s="7" t="n">
-        <v>48</v>
-      </c>
-      <c r="B49" s="8" t="inlineStr">
-        <is>
-          <t>14T4</t>
-        </is>
-      </c>
-      <c r="C49" s="9" t="inlineStr">
-        <is>
-          <t>Prestige 14 Flip AI+ D4MT</t>
-        </is>
-      </c>
-      <c r="D49" s="16" t="inlineStr">
-        <is>
-          <t>EVT</t>
-        </is>
-      </c>
-      <c r="E49" s="9" t="inlineStr">
-        <is>
-          <t>NVL-H 30W</t>
-        </is>
-      </c>
-      <c r="F49" s="9" t="inlineStr">
-        <is>
-          <t>Intel® Arc™ Graphics</t>
-        </is>
-      </c>
-      <c r="G49" s="9" t="inlineStr">
-        <is>
-          <t>朱芳芳</t>
-        </is>
-      </c>
-      <c r="H49" s="9" t="inlineStr">
-        <is>
-          <t>2026/05/14</t>
-        </is>
-      </c>
-      <c r="I49" s="9" t="inlineStr">
-        <is>
-          <t>2026/07/27</t>
-        </is>
-      </c>
-      <c r="J49" s="9" t="inlineStr">
-        <is>
-          <t>2026/10/17</t>
-        </is>
-      </c>
-      <c r="K49" s="9" t="inlineStr">
-        <is>
-          <t>2026/12/02</t>
-        </is>
-      </c>
-      <c r="L49" s="9" t="inlineStr">
-        <is>
-          <t>2026/12/30</t>
-        </is>
-      </c>
-      <c r="M49" s="9" t="inlineStr">
-        <is>
-          <t>2027/02/16</t>
-        </is>
-      </c>
-      <c r="N49" s="9" t="inlineStr">
-        <is>
-          <t>2027/02/26</t>
-        </is>
-      </c>
-      <c r="O49" s="11" t="inlineStr">
-        <is>
-          <t>EVT組裝中，DQA test12/26～11/16</t>
-        </is>
-      </c>
-      <c r="P49" s="11" t="inlineStr">
-        <is>
-          <t>PCB 1.0  for MVT 需采購pull in 11/30 ready (3W 進料,LT：4W）</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="n">
-        <v>49</v>
-      </c>
-      <c r="B50" s="3" t="inlineStr">
-        <is>
-          <t>2624</t>
-        </is>
-      </c>
-      <c r="C50" s="4" t="inlineStr">
-        <is>
-          <t>Prestige 16 AI+ C4M</t>
-        </is>
-      </c>
-      <c r="D50" s="15" t="inlineStr">
-        <is>
-          <t>EVT</t>
-        </is>
-      </c>
-      <c r="E50" s="4" t="inlineStr">
-        <is>
-          <t>NVL-H 30W</t>
-        </is>
-      </c>
-      <c r="F50" s="4" t="inlineStr">
-        <is>
-          <t>Intel® Arc™ Graphics</t>
-        </is>
-      </c>
-      <c r="G50" s="4" t="inlineStr">
-        <is>
-          <t>朱芳芳</t>
-        </is>
-      </c>
-      <c r="H50" s="4" t="inlineStr">
-        <is>
-          <t>2026/05/14</t>
-        </is>
-      </c>
-      <c r="I50" s="4" t="inlineStr"/>
-      <c r="J50" s="4" t="inlineStr">
-        <is>
-          <t>2026/10/17</t>
-        </is>
-      </c>
-      <c r="K50" s="4" t="inlineStr">
-        <is>
-          <t>2026/12/02</t>
-        </is>
-      </c>
-      <c r="L50" s="4" t="inlineStr">
-        <is>
-          <t>2026/12/30</t>
-        </is>
-      </c>
-      <c r="M50" s="4" t="inlineStr">
-        <is>
-          <t>2027/02/16</t>
-        </is>
-      </c>
-      <c r="N50" s="4" t="inlineStr">
-        <is>
-          <t>2027/02/26</t>
-        </is>
-      </c>
-      <c r="O50" s="6" t="inlineStr">
-        <is>
-          <t>EVT組裝中，DQA test12/26～11/16</t>
-        </is>
-      </c>
-      <c r="P50" s="6" t="inlineStr">
-        <is>
-          <t>PCB 1.0  for MVT 需采購pull in 11/30 ready (3W 進料,LT：4W）</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" hidden="1" outlineLevel="1">
-      <c r="A51" s="7" t="n">
-        <v>50</v>
-      </c>
-      <c r="B51" s="8" t="inlineStr">
-        <is>
-          <t>2624</t>
-        </is>
-      </c>
-      <c r="C51" s="9" t="inlineStr">
-        <is>
-          <t>Prestige 16 Flip AI+ C4MT</t>
-        </is>
-      </c>
-      <c r="D51" s="16" t="inlineStr">
-        <is>
-          <t>EVT</t>
-        </is>
-      </c>
-      <c r="E51" s="9" t="inlineStr">
-        <is>
-          <t>NVL-H 30W</t>
-        </is>
-      </c>
-      <c r="F51" s="9" t="inlineStr">
-        <is>
-          <t>Intel® Arc™ Graphics</t>
-        </is>
-      </c>
-      <c r="G51" s="9" t="inlineStr">
-        <is>
-          <t>朱芳芳</t>
-        </is>
-      </c>
-      <c r="H51" s="9" t="inlineStr">
-        <is>
-          <t>2026/05/14</t>
-        </is>
-      </c>
-      <c r="I51" s="9" t="inlineStr"/>
-      <c r="J51" s="9" t="inlineStr">
-        <is>
-          <t>2026/10/17</t>
-        </is>
-      </c>
-      <c r="K51" s="9" t="inlineStr">
-        <is>
-          <t>2026/12/02</t>
-        </is>
-      </c>
-      <c r="L51" s="9" t="inlineStr">
-        <is>
-          <t>2026/12/30</t>
-        </is>
-      </c>
-      <c r="M51" s="9" t="inlineStr">
-        <is>
-          <t>2027/02/16</t>
-        </is>
-      </c>
-      <c r="N51" s="9" t="inlineStr">
-        <is>
-          <t>2027/02/26</t>
-        </is>
-      </c>
-      <c r="O51" s="11" t="inlineStr">
-        <is>
-          <t>EVT組裝中，DQA test12/26～11/16</t>
-        </is>
-      </c>
-      <c r="P51" s="11" t="inlineStr">
-        <is>
-          <t>PCB 1.0  for MVT 需采購pull in 11/30 ready (3W 進料,LT：4W）</t>
         </is>
       </c>
     </row>
@@ -4405,12 +4385,12 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>14W2</t>
+          <t>2662</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Prestige 14S E4M</t>
+          <t>Prestige 16S D4M</t>
         </is>
       </c>
       <c r="D52" s="14" t="inlineStr">
@@ -4470,7 +4450,7 @@
       </c>
       <c r="O52" s="6" t="inlineStr">
         <is>
-          <t>0A layout中，预计10/22出图</t>
+          <t>10/22出图，DVT从11/4提前至10/31，后续schedule暂keep</t>
         </is>
       </c>
       <c r="P52" s="6" t="inlineStr">
@@ -4485,22 +4465,22 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>2662</t>
+          <t>13Q5</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Prestige 16S D4M</t>
-        </is>
-      </c>
-      <c r="D53" s="14" t="inlineStr">
-        <is>
-          <t>Design</t>
+          <t>Prestige 13 AI+ A4M</t>
+        </is>
+      </c>
+      <c r="D53" s="15" t="inlineStr">
+        <is>
+          <t>EVT</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>NVL-H 30W</t>
+          <t>NVL-H 28W</t>
         </is>
       </c>
       <c r="F53" s="4" t="inlineStr">
@@ -4510,47 +4490,47 @@
       </c>
       <c r="G53" s="4" t="inlineStr">
         <is>
-          <t>吳美芳</t>
+          <t>顏春梅</t>
         </is>
       </c>
       <c r="H53" s="4" t="inlineStr">
         <is>
-          <t>2026/09/11</t>
+          <t>2026/06/29</t>
         </is>
       </c>
       <c r="I53" s="4" t="inlineStr">
         <is>
-          <t>2026/10/31</t>
+          <t>2026/08/18</t>
         </is>
       </c>
       <c r="J53" s="4" t="inlineStr">
         <is>
-          <t>2026/12/13</t>
+          <t>2026/10/10</t>
         </is>
       </c>
       <c r="K53" s="4" t="inlineStr">
         <is>
-          <t>2027/01/14</t>
+          <t>2026/12/03</t>
         </is>
       </c>
       <c r="L53" s="4" t="inlineStr">
         <is>
-          <t>2027/01/21</t>
+          <t>2027/01/22</t>
         </is>
       </c>
       <c r="M53" s="4" t="inlineStr">
         <is>
-          <t>2027/02/18</t>
+          <t>2027/02/23</t>
         </is>
       </c>
       <c r="N53" s="4" t="inlineStr">
         <is>
-          <t>2027/02/28</t>
+          <t>2027/03/05</t>
         </is>
       </c>
       <c r="O53" s="6" t="inlineStr">
         <is>
-          <t>0A layout中，预计10/22出图</t>
+          <t>EVT 機台10/20調撥回台 預計23號 RD 開始測試</t>
         </is>
       </c>
       <c r="P53" s="6" t="inlineStr">
@@ -4620,22 +4600,22 @@
       </c>
       <c r="M54" s="4" t="inlineStr">
         <is>
-          <t>2027/03/08</t>
+          <t>2027/03/05</t>
         </is>
       </c>
       <c r="N54" s="4" t="inlineStr">
         <is>
-          <t>2027/03/18</t>
+          <t>2027/03/15</t>
         </is>
       </c>
       <c r="O54" s="6" t="inlineStr">
         <is>
-          <t>10/12组装，预计10/16调拨回台</t>
+          <t>EVT机台DQA test from 10/16, 调拨机台10/27到台北</t>
         </is>
       </c>
       <c r="P54" s="6" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>ATS pull in 3/5~3/15 Gating:1.WHQL GAP 6D,需pull in至3/4 ready  2.TBT  Signed FW Gap 2~3 weeks (PV BKC+3weeks) 需GRL&amp;Intel 幫忙</t>
         </is>
       </c>
     </row>
@@ -4700,22 +4680,22 @@
       </c>
       <c r="M55" s="9" t="inlineStr">
         <is>
-          <t>2027/03/08</t>
+          <t>2027/03/05</t>
         </is>
       </c>
       <c r="N55" s="9" t="inlineStr">
         <is>
-          <t>2027/03/18</t>
+          <t>2027/03/15</t>
         </is>
       </c>
       <c r="O55" s="11" t="inlineStr">
         <is>
-          <t>10/12组装，预计10/16调拨回台</t>
+          <t>EVT机台DQA test from 10/16, 调拨机台10/27到台北</t>
         </is>
       </c>
       <c r="P55" s="11" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>ATS pull in 3/5~3/15 Gating:1.WHQL GAP 6D,需pull in至3/4 ready  2.TBT  Signed FW Gap 2~3 weeks (PV BKC+3weeks) 需GRL&amp;Intel 幫忙</t>
         </is>
       </c>
     </row>
@@ -4780,22 +4760,22 @@
       </c>
       <c r="M56" s="9" t="inlineStr">
         <is>
-          <t>2027/03/08</t>
+          <t>2027/03/05</t>
         </is>
       </c>
       <c r="N56" s="9" t="inlineStr">
         <is>
-          <t>2027/03/18</t>
+          <t>2027/03/15</t>
         </is>
       </c>
       <c r="O56" s="11" t="inlineStr">
         <is>
-          <t>10/12组装，预计10/16调拨回台</t>
+          <t>EVT机台DQA test from 10/16, 调拨机台10/27到台北</t>
         </is>
       </c>
       <c r="P56" s="11" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>ATS pull in 3/5~3/15 Gating:1.WHQL GAP 6D,需pull in至3/4 ready  2.TBT  Signed FW Gap 2~3 weeks (PV BKC+3weeks) 需GRL&amp;Intel 幫忙</t>
         </is>
       </c>
     </row>
@@ -4865,7 +4845,7 @@
       </c>
       <c r="N57" s="4" t="inlineStr">
         <is>
-          <t>2027/03/18</t>
+          <t>2027/03/15</t>
         </is>
       </c>
       <c r="O57" s="6" t="inlineStr">
@@ -4945,7 +4925,7 @@
       </c>
       <c r="N58" s="9" t="inlineStr">
         <is>
-          <t>2027/03/18</t>
+          <t>2027/03/15</t>
         </is>
       </c>
       <c r="O58" s="11" t="inlineStr">
@@ -5025,7 +5005,7 @@
       </c>
       <c r="N59" s="9" t="inlineStr">
         <is>
-          <t>2027/03/18</t>
+          <t>2027/03/15</t>
         </is>
       </c>
       <c r="O59" s="11" t="inlineStr">
@@ -5105,7 +5085,7 @@
       </c>
       <c r="N60" s="9" t="inlineStr">
         <is>
-          <t>2027/03/18</t>
+          <t>2027/03/15</t>
         </is>
       </c>
       <c r="O60" s="11" t="inlineStr">
@@ -5185,7 +5165,7 @@
       </c>
       <c r="N61" s="9" t="inlineStr">
         <is>
-          <t>2027/03/18</t>
+          <t>2027/03/15</t>
         </is>
       </c>
       <c r="O61" s="11" t="inlineStr">
@@ -5265,7 +5245,7 @@
       </c>
       <c r="N62" s="9" t="inlineStr">
         <is>
-          <t>2027/03/18</t>
+          <t>2027/03/15</t>
         </is>
       </c>
       <c r="O62" s="11" t="inlineStr">
@@ -5320,7 +5300,11 @@
       </c>
       <c r="I63" s="4" t="inlineStr"/>
       <c r="J63" s="4" t="inlineStr"/>
-      <c r="K63" s="4" t="inlineStr"/>
+      <c r="K63" s="4" t="inlineStr">
+        <is>
+          <t>2027/01/11</t>
+        </is>
+      </c>
       <c r="L63" s="4" t="inlineStr">
         <is>
           <t>2027/02/02</t>
@@ -5328,12 +5312,12 @@
       </c>
       <c r="M63" s="4" t="inlineStr">
         <is>
-          <t>2027/03/08</t>
+          <t>2027/03/05</t>
         </is>
       </c>
       <c r="N63" s="4" t="inlineStr">
         <is>
-          <t>2027/03/18</t>
+          <t>2027/03/15</t>
         </is>
       </c>
       <c r="O63" s="6" t="inlineStr">
@@ -5343,7 +5327,7 @@
       </c>
       <c r="P63" s="6" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>ATS pull in 3/5~3/15 Gating:1.WHQL GAP 6D,需pull in至3/4 ready 2.TBT Signed FW Gap 2~3 weeks (PV BKC+3weeks) 需GRL&amp;Intel 幫忙</t>
         </is>
       </c>
     </row>
@@ -5388,7 +5372,11 @@
       </c>
       <c r="I64" s="9" t="inlineStr"/>
       <c r="J64" s="9" t="inlineStr"/>
-      <c r="K64" s="9" t="inlineStr"/>
+      <c r="K64" s="9" t="inlineStr">
+        <is>
+          <t>2027/01/11</t>
+        </is>
+      </c>
       <c r="L64" s="9" t="inlineStr">
         <is>
           <t>2027/02/02</t>
@@ -5396,12 +5384,12 @@
       </c>
       <c r="M64" s="9" t="inlineStr">
         <is>
-          <t>2027/03/08</t>
+          <t>2027/03/05</t>
         </is>
       </c>
       <c r="N64" s="9" t="inlineStr">
         <is>
-          <t>2027/03/18</t>
+          <t>2027/03/15</t>
         </is>
       </c>
       <c r="O64" s="11" t="inlineStr">
@@ -5411,7 +5399,7 @@
       </c>
       <c r="P64" s="11" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>ATS pull in 3/5~3/15 Gating:1.WHQL GAP 6D,需pull in至3/4 ready 2.TBT Signed FW Gap 2~3 weeks (PV BKC+3weeks) 需GRL&amp;Intel 幫忙</t>
         </is>
       </c>
     </row>
@@ -5458,7 +5446,7 @@
       <c r="J65" s="9" t="inlineStr"/>
       <c r="K65" s="9" t="inlineStr">
         <is>
-          <t>2026/11/11</t>
+          <t>2027/01/11</t>
         </is>
       </c>
       <c r="L65" s="9" t="inlineStr">
@@ -5468,12 +5456,12 @@
       </c>
       <c r="M65" s="9" t="inlineStr">
         <is>
-          <t>2027/03/08</t>
+          <t>2027/03/05</t>
         </is>
       </c>
       <c r="N65" s="9" t="inlineStr">
         <is>
-          <t>2027/03/18</t>
+          <t>2027/03/15</t>
         </is>
       </c>
       <c r="O65" s="11" t="inlineStr">
@@ -5483,7 +5471,7 @@
       </c>
       <c r="P65" s="11" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>ATS pull in 3/5~3/15 Gating:1.WHQL GAP 6D,需pull in至3/4 ready 2.TBT Signed FW Gap 2~3 weeks (PV BKC+3weeks) 需GRL&amp;Intel 幫忙</t>
         </is>
       </c>
     </row>
@@ -5528,7 +5516,11 @@
       </c>
       <c r="I66" s="9" t="inlineStr"/>
       <c r="J66" s="9" t="inlineStr"/>
-      <c r="K66" s="9" t="inlineStr"/>
+      <c r="K66" s="9" t="inlineStr">
+        <is>
+          <t>2027/01/11</t>
+        </is>
+      </c>
       <c r="L66" s="9" t="inlineStr">
         <is>
           <t>2027/02/02</t>
@@ -5536,12 +5528,12 @@
       </c>
       <c r="M66" s="9" t="inlineStr">
         <is>
-          <t>2027/03/08</t>
+          <t>2027/03/05</t>
         </is>
       </c>
       <c r="N66" s="9" t="inlineStr">
         <is>
-          <t>2027/03/18</t>
+          <t>2027/03/15</t>
         </is>
       </c>
       <c r="O66" s="11" t="inlineStr">
@@ -5551,7 +5543,7 @@
       </c>
       <c r="P66" s="11" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>ATS pull in 3/5~3/15 Gating:1.WHQL GAP 6D,需pull in至3/4 ready 2.TBT Signed FW Gap 2~3 weeks (PV BKC+3weeks) 需GRL&amp;Intel 幫忙</t>
         </is>
       </c>
     </row>
@@ -5616,22 +5608,22 @@
       </c>
       <c r="M67" s="9" t="inlineStr">
         <is>
-          <t>2027/03/08</t>
+          <t>2027/03/05</t>
         </is>
       </c>
       <c r="N67" s="9" t="inlineStr">
         <is>
-          <t>2027/03/18</t>
+          <t>2027/03/15</t>
         </is>
       </c>
       <c r="O67" s="11" t="inlineStr">
         <is>
-          <t>EVT DQA 測試中，台北機台10/16調撥，預計10/20 ETA</t>
+          <t>EVT  測試中</t>
         </is>
       </c>
       <c r="P67" s="11" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>ATS pull in 3/5~3/15 Gating:1.WHQL GAP 6D,需pull in至3/4 ready 2.TBT Signed FW Gap 2~3 weeks (PV BKC+3weeks) 需GRL&amp;Intel 幫忙</t>
         </is>
       </c>
     </row>
@@ -5696,22 +5688,22 @@
       </c>
       <c r="M68" s="9" t="inlineStr">
         <is>
-          <t>2027/03/08</t>
+          <t>2027/03/05</t>
         </is>
       </c>
       <c r="N68" s="9" t="inlineStr">
         <is>
-          <t>2027/03/18</t>
+          <t>2027/03/15</t>
         </is>
       </c>
       <c r="O68" s="11" t="inlineStr">
         <is>
-          <t>EVT DQA 測試中，台北機台10/16調撥，預計10/20 ETA</t>
+          <t>EVT  測試中</t>
         </is>
       </c>
       <c r="P68" s="11" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>ATS pull in 3/5~3/15 Gating:1.WHQL GAP 6D,需pull in至3/4 ready 2.TBT Signed FW Gap 2~3 weeks (PV BKC+3weeks) 需GRL&amp;Intel 幫忙</t>
         </is>
       </c>
     </row>
@@ -5776,22 +5768,22 @@
       </c>
       <c r="M69" s="9" t="inlineStr">
         <is>
-          <t>2027/03/08</t>
+          <t>2027/03/05</t>
         </is>
       </c>
       <c r="N69" s="9" t="inlineStr">
         <is>
-          <t>2027/03/18</t>
+          <t>2027/03/15</t>
         </is>
       </c>
       <c r="O69" s="11" t="inlineStr">
         <is>
-          <t>EVT DQA 測試中，台北機台10/16調撥，預計10/20 ETA</t>
+          <t>EVT 測試中</t>
         </is>
       </c>
       <c r="P69" s="11" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>ATS pull in 3/5~3/15 Gating:1.WHQL GAP 6D,需pull in至3/4 ready 2.TBT Signed FW Gap 2~3 weeks (PV BKC+3weeks) 需GRL&amp;Intel 幫忙</t>
         </is>
       </c>
     </row>
@@ -5856,22 +5848,22 @@
       </c>
       <c r="M70" s="9" t="inlineStr">
         <is>
-          <t>2027/03/08</t>
+          <t>2027/03/05</t>
         </is>
       </c>
       <c r="N70" s="9" t="inlineStr">
         <is>
-          <t>2027/03/18</t>
+          <t>2027/03/15</t>
         </is>
       </c>
       <c r="O70" s="11" t="inlineStr">
         <is>
-          <t>EVT DQA 測試中，台北機台10/16調撥，預計10/20 ETA</t>
+          <t>EVT 測試中</t>
         </is>
       </c>
       <c r="P70" s="11" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>ATS pull in 3/5~3/15 Gating:1.WHQL GAP 6D,需pull in至3/4 ready 2.TBT Signed FW Gap 2~3 weeks (PV BKC+3weeks) 需GRL&amp;Intel 幫忙</t>
         </is>
       </c>
     </row>
@@ -5951,7 +5943,8 @@
       </c>
       <c r="P71" s="6" t="inlineStr">
         <is>
-          <t>1.增加EVT-2 for NV機台（人力運送回台） 2.Fan&amp;CosMX 80Wh Re-Pack認證影響BSMI取證時間</t>
+          <t>1)增加EVT-2 for NV機台（人力運送回台）
+2)Fan&amp;CosMX 80Wh Re-Pack認證影響BSMI取證時間</t>
         </is>
       </c>
     </row>
@@ -6031,7 +6024,8 @@
       </c>
       <c r="P72" s="11" t="inlineStr">
         <is>
-          <t>1.增加EVT-2 for NV機台（人力運送回台） 2.Fan&amp;CosMX 80Wh Re-Pack認證影響BSMI取證時間</t>
+          <t>1)增加EVT-2 for NV機台（人力運送回台）
+2)Fan&amp;CosMX 80Wh Re-Pack認證影響BSMI取證時間</t>
         </is>
       </c>
     </row>
@@ -6111,7 +6105,8 @@
       </c>
       <c r="P73" s="11" t="inlineStr">
         <is>
-          <t>1.增加EVT-2 for NV機台（人力運送回台） 2.Fan&amp;CosMX 80Wh Re-Pack認證影響BSMI取證時間</t>
+          <t>1)增加EVT-2 for NV機台（人力運送回台）
+2)Fan&amp;CosMX 80Wh Re-Pack認證影響BSMI取證時間</t>
         </is>
       </c>
     </row>
@@ -6313,17 +6308,17 @@
       </c>
       <c r="I76" s="4" t="inlineStr">
         <is>
-          <t>2026/12/22</t>
+          <t>2027/01/05</t>
         </is>
       </c>
       <c r="J76" s="4" t="inlineStr">
         <is>
-          <t>2027/01/19</t>
+          <t>2027/01/26</t>
         </is>
       </c>
       <c r="K76" s="4" t="inlineStr">
         <is>
-          <t>2027/03/26</t>
+          <t>2027/04/08</t>
         </is>
       </c>
       <c r="L76" s="4" t="inlineStr">
@@ -6333,12 +6328,12 @@
       </c>
       <c r="M76" s="4" t="inlineStr">
         <is>
-          <t>2027/05/06</t>
+          <t>2027/05/18</t>
         </is>
       </c>
       <c r="N76" s="4" t="inlineStr">
         <is>
-          <t>2027/05/19</t>
+          <t>2027/05/29</t>
         </is>
       </c>
       <c r="O76" s="6" t="inlineStr"/>

</xml_diff>